<commit_message>
Shift conclusion section to SDM verification levels and default blank/empty numeric fields to 0 in reports/review tables
</commit_message>
<xml_diff>
--- a/patwari_reports.xlsx
+++ b/patwari_reports.xlsx
@@ -717,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DF6"/>
+  <dimension ref="A1:DJ10"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -1271,6 +1271,26 @@
           <t>sdm_dispatch_patwari_tehsil</t>
         </is>
       </c>
+      <c r="DG1" t="inlineStr">
+        <is>
+          <t>exam_passed_year</t>
+        </is>
+      </c>
+      <c r="DH1" t="inlineStr">
+        <is>
+          <t>diary_duty_compliance</t>
+        </is>
+      </c>
+      <c r="DI1" t="inlineStr">
+        <is>
+          <t>diary_duty_remarks</t>
+        </is>
+      </c>
+      <c r="DJ1" t="inlineStr">
+        <is>
+          <t>jinswar_submit_status</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -2371,7 +2391,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>2026-06-08T23:58:53.982125</t>
+          <t>2026-06-09T09:10:52.327175</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -2469,7 +2489,6 @@
           <t>सरकारी पटवार घर</t>
         </is>
       </c>
-      <c r="V5" t="inlineStr"/>
       <c r="W5" t="inlineStr">
         <is>
           <t>कोई नोटिस जारी नहीं।</t>
@@ -2500,7 +2519,6 @@
           <t>हस्ताक्षर लिये गये हैं</t>
         </is>
       </c>
-      <c r="AC5" t="inlineStr"/>
       <c r="AD5" t="inlineStr">
         <is>
           <t>0</t>
@@ -2673,7 +2691,7 @@
       </c>
       <c r="BL5" t="inlineStr">
         <is>
-          <t>{"rule116_status":"संधारित है","rule116_sign":"हस्ताक्षर लिये गये हैं","rule117_egras":"","copy_reg_status":"हाँ","store_reg_status":"हाँ","store_items_status":"पूर्ण","p37_reg_status":"हाँ","passbook_total_dist":"0","seeding_remarks":"","r91_active_count":"0","r91_inactive_count":"0","r91_overall_remarks":"","jinswar_remarks":"","rule121_pending_date":"2026-06-07","copy_remarks":"","store_remarks":"","passbook_remarks":"","r89_register_status":"संधारित की जा रही है","check_girdawari_remarks":"","dhal_samvat":"2081","dhal_year":"2024","recovery_not_started_count":"0","recovery_last_date":"","recovery_pending_start_date":"","recovery_pending_end_date":"","seamaprakaran_total_pending":"0","seamaprakaran_remarks":"","citizen_charter_register_status":"","grievances_register_status":"","rti_register_status":"","govt_schemes_progress":"","conclusion_text":"","sdm_dispatch_no":"","sdm_dispatch_date":"","sdm_dispatch_tehsil":"","sdm_dispatch_patwari_circle":"","sdm_dispatch_patwari_tehsil":"","cv_remarks":"","cc_remarks":"","al_remarks":"","ga_remarks":"","court_cases_remarks":"","nk_inst_custodian":"","nk_inst_allottee":"","nk_inst_settled":"","nk_inst_leaseholder":""}</t>
+          <t>{"rule116_status":"संधारित है","rule116_sign":"हस्ताक्षर लिये गये हैं","rule117_egras":"","copy_reg_status":"हाँ","store_reg_status":"हाँ","store_items_status":"पूर्ण","p37_reg_status":"हाँ","passbook_total_dist":"0","seeding_remarks":"","r91_active_count":"0","r91_inactive_count":"0","r91_overall_remarks":"","jinswar_remarks":"","rule121_pending_date":"2026-06-07","copy_remarks":"","store_remarks":"","passbook_remarks":"","r89_register_status":"संधारित की जा रही है","check_girdawari_remarks":"","dhal_samvat":"2081","dhal_year":"2024","recovery_not_started_count":"0","recovery_last_date":"","recovery_pending_start_date":"","recovery_pending_end_date":"","seamaprakaran_total_pending":"0","seamaprakaran_remarks":"","citizen_charter_register_status":"","grievances_register_status":"","rti_register_status":"","govt_schemes_progress":"","conclusion_text":"","sdm_dispatch_no":"","sdm_dispatch_date":"","sdm_dispatch_tehsil":"","sdm_dispatch_patwari_circle":"","sdm_dispatch_patwari_tehsil":"","cv_remarks":"","cc_remarks":"","al_remarks":"","ga_remarks":"","court_cases_remarks":"","nk_inst_custodian":"","nk_inst_allottee":"","nk_inst_settled":"","nk_inst_leaseholder":"","exam_passed_year":"","dhal_remarks":"","recovery_remarks":"","rule116_remarks":"","accidents_remarks":"","diary_duty_compliance":"हाँ","diary_duty_remarks":"","jinswar_submit_status":"समय पर पेश किये जाते हैं"}</t>
         </is>
       </c>
       <c r="BM5" t="inlineStr">
@@ -2683,14 +2701,9 @@
       </c>
       <c r="BN5" t="inlineStr">
         <is>
-          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAesAAACVCAYAAAB4rNKkAAAQAElEQVR4AezdD5RcVX3A8d99s5sQCDNDZHcmEBAlnLCzETnQoq3SQ6MtKqUqBf+hVUChp2Chta1Se1pOLYKn7TmlUC394xGp1vqvyp+CVFvACuVQBEx2NsEgmJPA7iaQmd0gbHbnXX935s26O26S2dmZN+/N+47vzr3v/+9+Lua3772ZXU94IYAAAggggECkBUjWkR4egkMAAQQQQEAkHsmakUIAAQQQQCDBAiTrBA8+XUcAAQQQiIcAybp948SREEAAAQQQ6IgAybojrBwUAQQQQACB9gmQrNtnGY8jESUCCCCAQOwESNaxGzICRgABBBBImgDJOmkjHo/+EiUCCCCAwDwBkvU8DJoIIIAAAghEUYBkHcVRIaZ4CBAlAgggEJIAyTokaE6DAAIIIIBAqwIk61bl2A+BeAgQJQII9IAAyboHBpEuIIAAAgj0tgDJurfHl94hEA8BokQAgYMKkKwPysNKBBBAAAEEui9Asu7+GBABAgjEQ4AoEeiaAMm6a/ScGAEEEEAAgeYESNbNObEVAgggEA8BouxJAZJ1Tw4rnUIAAQQQ6CUBknUvjSZ9QQABBOIhQJRLFCBZLxGMzRFAAAEEEAhbgGQdtjjnQwABBBCIh0CEoiRZR2gwCAUBBBBAAIHFBEjWi6mwDAEEEEAAgQgJHCRZRyhKQkEAAQQQQCDBAiTrBA8+XUcAAQQQiIdA7JN1PJiJEgEEEEAAgdYFSNat27EnAggggAACoQiQrENh5iQIIIAAAgi0LkCybt2OPRFAAAEEEAhFgGQdCnM8TkKUCDiB7EDhtkyu8Gg6N/S3bp6CAALdFyBZd38MiACByAik8ydfYz05VwM61Yi5MpMr/Pfq/PoBnWdCAIEuCpCsu4jPqVsRYJ9OChgruxqO/6t9dsXT2Vzh1oblzCKAQIgCJOsQsTkVAlEX0Kvp19RjNGLvdG0rcriW9x6VH3qLm6cggED4AiTr8M05YwIE4tjFzODGE62Y91ZjtzJTGj/87damavO6sGLN2VoxIYBAFwRI1l1A55QIRFDAGOPfr3Gt1CLWs28XeWRmcmLzF8TK3W6ZEXmXqykIIBC+AMk6fHPOiEBEBH4WRiZX+IwVOaa2xPzX5Nho9Ra4m7div+hqLYOZtcO/pTUTAgiELECyDhmc0yEQNYFMbuiNGtNlWkSvomdSM9MXV9vB2+RE7t+0uU+LrvffU615QwCBUAVI1qFyczIEoiWQOf5VR4mYmyV4eVY2Pf/89p3BbFDdO6uN2tW1NecdMVDI63xoEydCAAERkjX/FSCQZIHpikvUr3QERuxVe3cX/9e1G4s+z64la13R75l3a8WEAAIhCpCsQ8TmVAhESSCTH/6oxnOBFjHG3FoaH73BtRcrpbGt9xmRoltnra3dMnczlECACoHOCpCsO+vL0RGIpED1ObW117vgXBJe3Vc+ZAKuiNSuuo1sSK8dutLtS0EAgXAESNbhOHOWhAhkcsNfyuQKm7ODhX+Napcbn1MbXy7buXPni4eM1/q31LcxvvmTNWvWp+vz1PEQIMr4CpCs4zt2RB4xgUx+SG8r23dqWButkQuzg0Nv03b0piafUzcGPjWx9QF9rv37wfJBv3/Fp4M2FQIIdFiAZN1hYA6fIAFfjl/QW2t+vGA+AjNLeU69WLjBc+2H3TorcmE6X3iza1MQaJ8AR1pMgGS9mArLEGhFwJjTFuzmmbMWzHd5ppXn1IuEbMV67tPgL7l1xsrnuB3uJCgIdFaAZN1ZX46eFIETTjhMu3qGlrnJVvz75ma63Gj5OfUicZcntjypt8OvDlZxOzyAoEqWQNi9JVmHLc75elIg89KqD2vHFvz/yRjj67IoTEamK/+pgRzy+9S6TVMTt8ObYmIjBNomsOAfl7YdlQMhkDABa+1xjV22YtY3LuvGfDY/7D7F/Vp3bmPka0GidbPLKdwOX44e+yKwRIHWkvUST8LmCPS6gBHZ3NhHvVX8ZOOysOfXHHvKOrH++dXzWlvpm61cVG234Y3b4W1A5BAINClAsm4Sis0QOJiAsWZ343q9sj6xcVnY87OzszdpHKvceY3nXbJnz7Yp125XCa7S+XR4u0A5DgIHEOjlZH2ALrMYgXAEun1l7b7nrVf8b6311t5bGhtxt8Nrs+1753Z4+yw5EgIHFCBZH5CGFd0QyA4WPpIZLBzyV192I7alnlOvaLt2ZT0wUFit578xiHlaxL84aLe94nZ420k5IAI/J0Cy/jmSkBdwujmBdH7oHGvkr8XIPxyVG9o4tyIODSOnN4bZzSvrac/8pTquczFZK9eVx7c95dqdKtwO75Qsx0WgJkCyrjnwHgEBz5f+ehjWN331dhxqvRe8Y5E47SLLOr4os/bk0/X29xXVE1nZNjkxeG213dk3JeCXpXSWmKMnWYBkneTRb77vYW2pOSasU7X3PAf4gFkXvrq1fqX43ldFbMr10Bf/IpF7Z12706Xxdnilf8XXO31Ojo9AUgRI1kkZ6Vj005u79W0ldVIsQg6CtOJVk2MwW62M2JC/unVWXzbff4+e/AQtbvrK1MTWB10jrOJuh+vthNHgfG/IDgy/P2hTIYDAMgRI1svAY9c2C/Tb2/WI+m+9uy6suN8IprNLmLq4qd4SKCxy+mpfFlnegUVn9aVzE1+11vyKO7ieeFpeSnXjg3q2z/ofdDG4Yo1/7bp166pfHXPzFAQQaE2AZN2aG3t1QKC0q/iYGNFbuCLGypnZtUPVxCMxeNmU536dZ5ci1Svq3O5v6A8Mwde05OGVvhxdLm/e242Anp/Y+oAx9hPVcxtz7NRsutauLuANAQRaESBZt6LGPh0T0Muyj+vB9cJQxPfNR7Qdi6n87OZHNNAFf7jDLv7rRnWzdk61RG3FnhMc9eEVvmzavbu4L5jvSlVaPXOtiHlK3Muaq2L36X4XNwWBCAmQrCM0GIQiMrlz9Iea5G5wFnqleO7q/PBit5fd6sgVjfvR+UF1/pl1NBN11WD79mljTPDdbpvyrfmcLjdamBBAoAUBknULaOzSWQGbcldl8qKexaSsfFbrWEyeqbgfMuy8YOe35y1uR7PDiboNIZbGttwrYr4k7mXk9Mxg4VLXpCCAwNIFSNZLN2OPDgtMPfPEHn12fUftNPY1mVzh5lo72u+lsa1PWzFB3Bqr8ap/klJbbZ6in6jrHfb7Ku773rVb8kauP/LYk19WX0eNAALNC5Csm7diyxAFPE/+UBP2/uCUl2YHh24K2pGuPOtXPyDngrSe756/u2YbS3wStev01K6tz1ljP+raWrKpWc/dfdBmWyYOgkBiBEjWiRnqeHV07zPFHbO+d7xG/SMtYo25PJMb+kfXjniZnIvPymnpfOHubP7k+vee51a11ohXoq73cXJs9DNixX0ATyu5MJvfeFZ9HTUCCDQnQLJuzomtuiDwwsSW8Vnr/bKeupqwRcyHop+wvVfJvJexcra13rb0YOHPZf36lfNWLal55NEbNmTy44/O+9T3Q1H41HeTnbCesR8QMRXRl7X2s8ux0EPEayJaBNogQLJuAyKH6JxA3BK29WR1XcMY475f7D4ot8IYuSYztWIsM1i4OZ0fekszV9uZwY0npnNDf5rJFR71UqmtYs3G6rGtfF8T9Ru7/fWsaixNvu0dH91ixf+72ub2FenJFR+rtXlHAIFmBEjWzSixTVcFqgnbl9dpENu16GQ+lM4VvqCN6E1WXh4Etas0NvJn/ZXKen32/rVgWVbblxpr7tSr7ac0CZe1PKjloUxu+J5MrvDJTG74+kyu8O1MvrBDjL/dSDXhnxrs76q9ft/s2XFK1C5oV9L9U+4Z/phr6w8vV2dyG17h2pRICBBExAVI1hEfIMKrCbywuzg268uZRmSXW6L1ezK5oUtcO1rFnhLE87ir9+zZ9kx5rHi+WPkdEVu9DeyWByWt9Wu1nKHrfk3rq7V2H8Z6g25/nM7Xp+dEzL9Ya95UHi8OVD8tL/F77dy580Vj7e8Gka8U8WLztbwgZioEuiZAsu4aPSdeqoBL2JVK/yaxZqa2r7kpOzj86lo7Au+FwgqNYoMWN/3AvdVLeaJ4c3l8tE+fweeNMZusMVdoPz6tyfn/tLgkbnXb6aBo21b02e4tYr2zy+PFXHl85IOTEyPf0vVuW63iOZUmRv9D7y64fmgHzFn6LP9CbTAh0JxAgrciWSd48OPY9ak9jz+hz4XdLXGX2A6zxt6+Or9+IAp9yez13YfLqv+fsmKrV9aNcblb+qWxkf+ZHBv5+/LEyOXl8dFf0tJXHi96Wg4LirZH+yYnRj9Qntji/opWrBN0o0Eq1ef+0Id7li/GyA3Z7KnZxm2YRwCBhQLVf1gWLmIOgWgLaKJ7WIy8L4jyuJRdcacs45PWwXGWXRnfe3X9IL7xFlxZ15dTizy/6wc7xdhrAouX2ZX7rw/aVAj0gkBH+kCy7ggrB+20QHms+BU9x3Va3PSLmakVt7pGN4svpv68ev++sZGt3Ywl6ucuj43+jVjZFsR5aWbtyacHbSoEEFhEgGS9CAqL4iGgt4w/bkVuC6K9IJ0brreDReFWRvzalbWVzXpmXwvTgQUqvvgXBauVznN/6CMVzFMhgECDgNcwv+xZDoBAiAI23T/5Lr1CCz4hbs/N5AtfXrdu3aoQY5h3KlNL1ka4BT5P5UDNqYmtD4rYfwrWb8wOFq4K2lQIINAgQLJuAGE2XgLu60B91d+OZWsfwrJywb6Z9P8fNVB4fZg9WXPsKev0fEdp0cfpdtEPl7l1lIUCZnrlH+uS57SINfKJwNHNUhBAYJ5AQpP1PAGasRd4bnz027Kyz30i3D3HFr01XvA9+W4mxL/W5c/OnleHtCb1bL1NfXCBUumxkrH2D4KtVs1WZu8O2lQIIDBPgGQ9D4NmfAXKOzbv1WfY7xBj5v8ay0szueFvSe37zx3tnP6AMBycwJYzM3cFbaomBEoTo583Yqq/nc5YGU7nhq5sYjc2QSBRAiTrCA83oS1doDw28inx5Z0S/NEIfSb665nn7PeOPnrDMdLZ15nB4e+SbdumgjZVkwLWVi7XWyL6M4+IJu7rVueHC8ILAQTmBEjWcxQ0ekWgvLv45VRf6gT9x7/6ZxlFzC/MpFKP6RWb+9We0u5X8Jx1yB1Xn7tyVe0glljKE1vvEc/9kFXdcZUn9uZqizcEEKgKkKyrDLy1LhDNPd0v3iin97/OGFP//vWAXrHdn84Xrmh3xJWZ2d+oH7Mv1feNept6aQLl6nfn7afcXno7/PU6Vve7NgUBBER/lkUBgV4V2L59ujQ28tt6tfth7eKsln5NAjdm88Ofb+dzbD3+m/XYovdvn3A/JAivlgXK46MfM0ZG3AF0rM5MDw79hWtTEEi6AFfWSf8vIAH9nxwr3uR5skm7uluLWGvfl9kjDxx+9NBaN7/MktLb7dVkba25a5nHYncVsFauFKv/07YY80c8v3YQpctk4AAABbZJREFUlKQLkKyT/l9AQvq/99nid1N9fadpCqg9xzZyen/KPL7c59i6/1/plWC/YzTW7nQ1ZXkC5fHidyR4fm1EDuP59fI82bs3BEjWvTGO9KIJAXeL2j3H1ivrW4LN3XPs72VyhX9fc8zG+X8/Olh98OrIYzZsMOL9ntReL5n9P/nnWrPVd/arC5Qbn1/nhr9ZX0eNQBIFSNZJHPUk91mfY7s/PWlFXJJ1v7/b/X/gHZWKvyOTG/5hJjf0xWYTtzebul3EphynNfb8UunpkmtT2iNQ1ufXYqR6J8SI/c0jB4bf354jcxQE4ifg/qGKX9REjMAyBSbHizfqLdbzNNnWfk1p9Xh2vYh5t0vc2Vzh6Wxu+I5MrvCdzGDhrnn1J7XtypOaSE4SfRljvz45NnqnNhMxhdlJfX59ef18xrP8Za46BnXiBEjWiRtyOlwXKI0Xv1k+cuYITdpv0yvt2zRxa1Vbq42XW7Hn6NwmTcpvmldfrW1XXqm16Lr9lRcOv0x4dURAf6h6SA98nxallotdTUEgiQIk6ySOOn3+mYDeFndJW5PCWzVxr3KJ24i5QzfQXC3uNrmrNXdLvZ4WY/ZX58S8MDNrT5iaemSPbs/UIQGF3xcc+og1uQ2XBO1DVKxGoLcESNa9NZ70ZjkCQeIujY+cWx4veuWJYiqovXn1YeWxkZW6TpeNrP7JnlH+aMdyzJvYN2XM3B/3mJXUliZ2YRMEek6AZN1zQ0qHEOgtAevbua/Eeb5M91Lv6AsCzQqQrJuVYjsEEOiKgOkz39cTu7/K9XBpd/FxbTMhkDgBknXihpwOIxAvgb3PFHfoY4iTtJyhkbvPD2jFFJ4AZ4qCAMk6CqNADAgggAACCBxEgGR9EBxWIYAAAgjEQ6DXoyRZ9/oI0z8EEEAAgdgLkKxjP4R0AAEEEEAgHgKtR0mybt2OPRFAAAEEEAhFgGQdCjMnQQABBBBAoHWBMJN161GyJwIIIIAAAgkWIFknePDpOgIIIIBAPARI1o3jxDwCCCCAAAIREyBZR2xACAcBBBBAAIFGAZJ1o0g85okSAQQQQCBBAiTrBA02XUUAAQQQiKcAyTqe4xaPqIkSAQQQQKAtAiTrtjByEAQQQAABBDonQLLunC1HjocAUSKAAAKRFyBZR36ICBABBBBAIOkCJOuk/xdA/+MhQJQIIJBoAZJ1ooefziOAAAIIxEGAZB2HUSJGBOIhQJQIINAhAZJ1h2A5LAIIIIAAAu0SIFm3S5LjIIBAPASIEoEYCpCsYzhohIwAAgggkCwBknWyxpveIoBAPASIEoEFAiTrBRzMIIAAAgggED0BknX0xoSIEEAAgXgIEGVoAiTr0Kg5EQIIIIAAAq0JkKxbc2MvBBBAAIF4CPRElCTrnhhGOoEAAggg0MsCJOteHl36hgACCCAQD4FDREmyPgQQqxFAAAEEEOi2AMm62yPA+RFAAAEEEDiEQESS9SGiZDUCCCCAAAIJFiBZJ3jw6ToCCCCAQDwESNZLGCc2RQABBBBAoBsCJOtuqHNOBBBAAAEEliBAsl4CVjw2JUoEEEAAgV4TIFn32ojSHwQQQACBnhMgWffckMajQ0SJAAIIINC8AMm6eSu2RAABBBBAoCsCJOuusHPSeAgQJQIIIBANAZJ1NMaBKBBAAAEEEDigAMn6gDSsQCAeAkSJAAK9L0Cy7v0xpocIIIAAAjEXIFnHfAAJH4F4CBAlAggsR4BkvRw99kUAAQQQQCAEAZJ1CMicAgEE4iFAlAhEVYBkHdWRIS4EEEAAAQQCAZJ1AEGFAAIIxEOAKJMoQLJO4qjTZwQQQACBWAmQrGM1XASLAAIIxEOAKNsrQLJurydHQwABBBBAoO0CJOu2k3JABBBAAIF4CMQnSpJ1fMaKSBFAAAEEEipAsk7owNNtBBBAAIF4CLgoSdZOgYIAAggggECEBX4KAAD//0bq1tIAAAAGSURBVAMAqeTWZyxe0/8AAAAASUVORK5CYII=</t>
-        </is>
-      </c>
-      <c r="BO5" t="inlineStr"/>
-      <c r="BP5" t="inlineStr"/>
-      <c r="BQ5" t="inlineStr"/>
-      <c r="BR5" t="inlineStr"/>
-      <c r="BS5" t="inlineStr"/>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAfEAAACVCAYAAABIIMOFAAAPZklEQVR4AezdXYyc11kH8PPOui2BeGdNXY/bhCZNArZ3nRYQiEit1FxwARKUr1YigFoumiI1SEAkKBItFxQhggrpBeUi4YIgJSARUAtI9AaplVKpgRZKtN1xUzsY0Y+dTerurNMotb3z9jnbdZPWsbsfM/N+zG/1np3dMzPvc87vJP5nz9nIneSDAAECBAgQaKSAEG/kshk0AQIECBBIqZoQJ0+AAAECBAjsW0CI75vQDQgQIECAQDUCsxTi1QirSoAAAQIEJiQgxCcE67YECBAgQGDSAkJ80sLuT4AAAQIEJiQgxCcE67YECBAgQGDSAkJ80sLV3F9VAgQIEJgBASE+A4tsigQIECDQTgEh3s51rWZWqhIgQIDAVAWE+FS5FSNAgAABAuMTEOLjs3SnagRUJUCAwMwKCPGZXXoTJ0CAAIGmCwjxpq+g8VcjoCoBAgRqICDEa7AIhkCAAAECBPYiIMT3ouY9BKoRUJUAAQLfJiDEv43DNwQIECBAoDkCQrw5a2WkBKoRUJUAgdoKCPHaLo2BESBAgACBawsI8Wv7eJYAgWoEVCVAYAcCQnwHSF5CgAABAgTqKCDE67gqxkSAQDUCqhJomIAQb9iCGS4BAgQIELgsIMQvS3gkQIBANQKqEtizgBDfM503EiBAgACBagWEeLX+qhMgQKAaAVVbISDEW7GMJkGAAAECsyggxGdx1c2ZAAEC1QioOmYBIT5mULcjQIAAAQLTEhDi05JWhwABAgSqEWhxVSHe4sU1NQIECBBot4AQb/f6mh0BAgQIVCMwlapCfCrMihAgQIAAgfELCPHxm7ojAQIECBCYisAVIT6VqooQIECAAAEC+xYQ4vsmdAMCBAgQIFCNQE1CvJrJq0qAAAECBJosIMSbvHrGToAAAQIzLTDTIT7TK2/yBAgQINB4ASHe+CU0AQIECBCYVQEhPvWVV5AAAQIECIxHQIiPx9FdCBAgQIDA1AWE+NTJqymoKgECBAi0T0CIt29NzYgAAQIEZkRAiM/IQlczTVUJECBAYJICQnySuu5NgAABAgQmKCDEJ4jr1tUIqEqAAIFZERDis7LS5kmAAAECrRMQ4q1bUhOqRkBVAgQITF9AiE/fXEUCBAgQIDAWASE+FkY3IVCNgKoECMy2gBCf7fU3ewIECBBosIAQb/DiGTqBagRUJUCgLgJCvC4rYRwECBAgQGCXAkJ8l2BeToBANQKqEiBwpYAQv9JEDwECBAgQaISAEG/EMhkkAQLVCKhKoN4CQrze62N0BAgQIEDgqgJC/Ko0niBAgEA1AqoS2KmAEN+plNcRIECAAIGaCQjxmi2I4RAgQKAaAVWbKCDEm7hqxkyAAAECBEJAiAeCiwABAgSqEVB1fwJCfH9+3k2gVQIHDx//oVZNqCaT6fZuv6UmQzGMlgkI8ZYtqOkQ2KvAwpETP9+Z63yu21s8O99bumuv9/G+FwQWjh6/uXtk8R9S2jwz31v88AvP+KpagfZUF+LtWUszIbAvgTIVt23f4KYilY8s9BYf67765I9t93nYhUD3tbcfmu+d+Iuy7PxvKtJb81uLlPw0niG0sQoI8bFyuhmB5goM11Y+EKP/g2jPRUtlSm9Mo9F/dnsnHvn+15z8gdynfXeBhSOL96avb54pUvE7L3r1h4tO+bMv+t6XMygwiSkL8UmouieBhgoMByt/sllcuDml8sGUis209VHctbk5+nz3yNJ9hw8fO7jV5dMVAt2jS2/t9hZPl0X683jyULR8LY/K4k3h+gvrX+7/X+7QCIxTQIiPU9O9CLRA4NnV008PB/13bXaK22Mr+KPbU3pFKsrfuzg399T80aV7UrrzwHb/zD/kI4cI70+msoyz73TrFkiZvlCU5TuGg5XXn1/77Ce2+nwiMAGBzne9pxcQIDCTAs9+ebk/XF356aIY3RkA/Wj5Ohzh9JfdI2vLC72lt+SOWW35iKHbW/q7OHL4jzD4iWj5erZM5fuG3/vcD66v9f82OuJUIj67CExIQIhPCNZtCbRFYH311MfjJ8qTscV+d8xpNVqKn9CPRVh9ZKG3+Nih3ol4Ls3MRz5SyEcL+YghTH45Jl6kVMTRQ/lgHEXcsjHo/3E6e/b55IPAFATqGuJTmLoSBAjsQmA0HPT/+nvSgduKonx/vO9bv/w2SsUTscX+UITba6K/xdedB2Ke9+QjhXy0EBN9RbQU/0Hz0Xz0ED7vejaOIpIPAlMUEOJTxFaKQNMFBoMnvra+2v/DS2XnlrIsH4r5jKJFrpdvj3A7vdBben+v9/rvi75WXTGvt+QjhHyUEBM7HC1f/SKOGoZx5JCPHnKHRmDaAkL8xeK+JkBgRwJfW1sebKz1f72TyjfEXvLlX9y6LrbY3/t8unQmzorz1nvj/3w5FEcFC3FkEPP6SPzEfWwbJ44UyruHg5WT63HUsN3ngUAlAo3/l6wSNUUJENgS+Oqgv7w+WHnTKHXy/wN9aqszpV6cFT/Q7S3+z/yrln5qu69RD/loILbOHxrFUUGZ0hu3B/9cEUcJ+UhhGEcL0TeK5iJQqYAQr5R/q7hPBBovcH6w/K/D+Mm0LMp7YjJPR8vXyaJT/luE+ceuf/XJE7mj7q0XRwELcSSQjwZi6/ztMd7YaEijfHSQjxDyUUI+Uoh+F4FaCAjxWiyDQRBohcDmxmr/r162uXlr/CR+X8zo8m9ov3luNFru9pYevP7oba+K/jpenRjf3fkoILbO3xsDvC5a7KCnT+Qjg3x0kI8Qcp9GoE4CQrxOqzHNsahFYEICzzzzufPDQf/35+Y6+W9EeyTKxI50ij9rynfOlS9/av7I0vtuvPHGrZCM5yq/8pZ/N7b+4z88HojBxFFAfE7p1CiOCPJRQT4y2OrxiUANBeJfrBqOypAIEGi8wLkvLf//cLDyq8Uo/WhM5vFo+bo+zpX/6PzF+c8vHF16R3Tk7ep4mP6Vt/gjvD+Wt/yj+uX/1/3pfCQQ4z6Zjwii30Wg1gJCvNbL07rBmdAMCqw/vfKZCMU7irLzSzH909HydUOcM/9NhOgTB48sXf7Fsdw/8Za39LuxtZ+3+KPYm6PlK7b+y/vyUUA+EoiOzWguArUXEOK1XyIDJNAOgfW15X8aDq5bLFKZ/3avc9uzOtkpyscWeif+5eDh43n7fbt7/A95Cz9v5c/Fln5snb8zKuQ//8p4fGQutv6HcQSQjwLiexeBxgjkf4gbM1gDJbAnAW+qkcCnL64P+h+cu3jhdWUq74+BXYiWylT8TGeu89nukaUPHbzh+Ctz3xhbkbfu8xZ+3sqP+14fLV+P563+YWz5563/3KERaJqAEG/aihkvgRYInDt3emNj0L+3KEbHIsEf3Z7SgVSU7+5c6jzVPbr0nrS4+PLt/j0/5K36bm/xibx1Hze5IVq+ThextR/hfUfe6s8dGoGmCgjxpq6ccdddwPh2ILC+eurscG3lbWVKd8QW96e23zKfyvJPu19JT873ln4l+nb9y295az5v0eet+nj/5V9aO5e38vOW/nps7Ue/i0DjBYR445fQBAg0X2BjsPL4cND/8TKVd8VszkbL100Rug/HT9L/Nd9bvPxXfeb+q7a8FZ+35PPWfBlb9NsvvBD3vT9v4eet/JQ+fXG73wOBxgsI8cYvoQkQeJFAw7/cGPT/fvjKdCy21d+TUhpGy9cPx4/in+wePfGPC0eP35w7rmix9Z634PNWfLz33fH8gWjxw316NG/Zx33vzVv4W30+EWiRgBBv0WKaCoFWCKysXBiu9v9sdGB0a1GWH4o5XYoWgVz8Yll28hb7/d3X3n5oqy+lYj623PPWe96CTynNR4ur/FQZW/TD2KrPW/bR4SLQSgEh3splNSkCUxWYSLHzXzz1lfW1/m+msnM8Avmft4u8LLbYfzt9ffNMhPcHY6v9v+P7h+O5m6Ll62xsnd+Vt+Y3Yos+d2gE2iwgxNu8uuZGoAUCw7XlMxHIPxfb4nfGdD4TLV+HIrx/K754Q7R8DVOZfnc4WHndRmzJ5w6NwCwICPFZWGVzJNACgdgW/3iE9I+UZfq1+Ml8mF6Y0wOjuUu3xdb5B17o8hWB2RAQ4rOxzmZJoDUCG2srD29c99zRUZEeTQcu/WQE+2+c/9KTz7RmgiZCYBcCQnwXWF5KgEBNBM6eff786srbhl988t+nPCLlCNRKQIjXajkMhgABAgQI7FxAiO/cyisJECBQjYCqBK4iIMSvAqObAAECBAjUXUCI132FjI8AAQLVCKjaAAEh3oBFMkQCBAgQIPBSAkL8pVT0ESBAgEA1AqruSkCI74rLiwkQIECAQH0EhHh91sJICBAgQKAagcZWFeKNXToDJ0CAAIFZFxDis/5PgPkTIECAQDUCY6gqxMeA6BYECBAgQKAKASFehbqaBAgQIEBgDAJ7CPExVHULAgQIECBAYN8CQnzfhG5AgAABAgSqEWhMiFfDoyoBAgQIEKivgBCv79oYGQECBAgQuKaAEL8mjycJECBAgEB9BYR4fdfGyAgQIECAwDUFhPg1eap5UlUCBAgQILATASG+EyWvIUCAAAECNRQQ4jVclGqGpCoBAgQINE1AiDdtxYyXAAECBAhsCwjxbQgP1QioSoAAAQJ7FxDie7fzTgIECBAgUKmAEK+UX/FqBFQlQIBAOwSEeDvW0SwIECBAYAYFhPgMLropVyOgKgECBMYtIMTHLep+BAgQIEBgSgJCfErQyhCoRkBVAgTaLCDE27y65kaAAAECrRYQ4q1eXpMjUI2AqgQITEdAiE/HWRUCBAgQIDB2ASE+dlI3JECgGgFVCcyegBCfvTU3YwIECBBoiYAQb8lCmgYBAtUIqEqgSgEhXqW+2gQIECBAYB8CQnwfeN5KgACBagRUJfBNASH+TQefCRAgQIBA4wSEeOOWzIAJECBQjYCq9RMQ4vVbEyMiQIAAAQI7EhDiO2LyIgIECBCoRkDVawkI8WvpeI4AAQIECNRYQIjXeHEMjQABAgSqEWhKVSHelJUyTgIECBAg8B0CQvw7QHxLgAABAgSqEdh9VSG+ezPvIECAAAECtRAQ4rVYBoMgQIAAAQK7FxhHiO++qncQIECAAAEC+xYQ4vsmdAMCBAgQIFCNQHNDvBovVQkQIECAQG0EhHhtlsJACBAgQIDA7gSE+O68vJoAAQIECNRGQIjXZikMhAABAgQI7E5AiO/Oq5pXq0qAAAECBF5CQIi/BIouAgQIECDQBAEh3oRVqmaMqhIgQIBAzQW+AQAA//+u4aJwAAAABklEQVQDAAyunUnkvanfAAAAAElFTkSuQmCC</t>
+        </is>
+      </c>
       <c r="BT5" t="inlineStr">
         <is>
           <t>Pending</t>
@@ -2713,13 +2726,9 @@
       </c>
       <c r="BX5" t="inlineStr">
         <is>
-          <t>{"remarks":"कोई विशेष कमी नहीं पाई गई।","status":"समय पर","jan":"","feb":"","mar":"","apr":"","may":"","jun":"","jul":"","aug":"","sep":"","oct":"","nov":"","dec":""}</t>
-        </is>
-      </c>
-      <c r="BY5" t="inlineStr"/>
-      <c r="BZ5" t="inlineStr"/>
-      <c r="CA5" t="inlineStr"/>
-      <c r="CB5" t="inlineStr"/>
+          <t>{"remarks":"कोई विशेष कमी नहीं पाई गई।","status":"समय पर","jan":"60105-02-20","feb":"60204-02-20","mar":"","apr":"","may":"","jun":"","jul":"","aug":"","sep":"","oct":"","nov":"","dec":""}</t>
+        </is>
+      </c>
       <c r="CC5" t="inlineStr">
         <is>
           <t>संधारित है</t>
@@ -2740,14 +2749,11 @@
           <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAeoAAACWCAYAAAAR+ss0AAAIY0lEQVR4AezVMW4bRxgFYCZlmhQpDPgIbl34Vulzg/Q5UhqfQFcIDARIXLm0SViGTVsiudyd2Xnzf4ZoSeTuzJvvp/h+PvhHgAABAgQIDCugqIcdjWAECBAgQOBwyCpqEyNAgAABAsUEFHWxgTsuAQIECGQJKOp287IyAQIECBBYLaCoVxNagAABAgQItBNQ1O1ss1aWlgABAgSGFFDUQ45FKAIECBAg8FlAUX928H+WgLQECBAoI6Coy4zaQQkQIEAgUUBRJ05N5iwBaQkQILBCQFGvwHMrAQIECBBoLaCoWwtbn0CWgLQECAwmoKgHG4g4BAgQIEDgWwFF/a2GnwkQyBKQlkABAUVdYMiOSIAAAQK5Aoo6d3aSEyCQJSAtgbsEFPVdbG4iQIAAAQJ9BBR1H2e7ECBAIEtA2mEEFPUwoxCEAAECBAj8KKCofzTxDAECBAhkCUydVlFPPV6HI0CAAIF0AUWdPkH5CRAgQCBLYGFaRb0QzOUECBAgQKCngKLuqW0vAgQIECCwUGDnol6Y1uUECBAgQKCYgKIuNnDHJUCAAIEsAUW9YF4uJUCAAAECvQUUdW9x+xEgQIAAgQUCinoBVtal0hIgQIDADAKKeoYpOgMBAgQITCugqKcdbdbBpCVAgACBpwUU9dMuniVAgAABAkMIKOohxiBEloC0BAgQ6CegqPtZ24kAAQIECCwWUNSLydxAIEtAWgIEsgUUdfb8pCdAgACByQUU9eQDdjwCWQLSEiDwvYCi/l7E7wQIECBAYCABRT3QMEQhQCBLQFoCPQQUdQ9lexAgQIAAgTsFFPWdcG4jQIBAloC0qQKKOnVychMgQIBACQFFXWLMDkmAAIEsAWm/CijqrxZ+IkCAAAECwwko6uFGIhABAgQIZAm0Tauo2/panQABAgQIrBJQ1Kv43EyAAAECBNoKbF3UbdNanQABAgQIFBNQ1JMM/OXL17/8+uLV2+PjX49XDF4wKPp38Pb0WTDJx5pjPArULupHhBm+ffj44fXxHG+Oj988DgwODIr+Hbx5/Cw4Ht/XLAKKepJJ/vfPw9/Ho/zx0+HwlwcD74Ga74HTZ8DjZ8HxR1+zCCjqnEleTfr+3cOf/797+N2DgfdAzffA6TPg6geFC+IEFHXcyAQmQIAAgUoCirrStHue1V4ECBAgsImAot6E0SIECBAgQKCNgKJu42rVLAFpCRAgMKyAoh52NIIRIECAAIHDQVF7FxBIE5CXAIFSAoq61LgdlgABAgTSBBR12sTkJZAlIC0BAisFFPVKQLcTIECAAIGWAoq6pa61CRDIEpCWwIACinrAoYhEgAABAgS+CCjqLxK+EyBAIEtA2iICirrIoB2TAAECBDIFFHXm3KQmQIBAloC0dwso6rvp3EiAAAECBNoLKOr2xnYgQIAAgSyBodIq6qHGIQwBAgQIEDgXUNTnHn4jQIAAAQJDCVwt6qHSCkOAAAECBIoJKOpiA3dcAgQIEMgSmKyos/ClJUCAAAEC1wQU9TUhrxMgQIAAgR0FFPWO+LYmQIAAAQLXBBT1NSGvEyBAgACBHQUU9Y74WVtLS4AAAQJ7CCjqPdTtSYAAAQIEbhRQ1DdCuSxLQFoCBAjMIqCoZ5mkcxAgQIDAlAKKesqxOlSWgLQECBB4XkBRP2/jFQIECBAgsLuAot59BAIQyBKQlgCBvgKKuq+33QgQIECAwCIBRb2Iy8UECGQJSEsgX0BR58/QCQgQIEBgYgFFPfFwHY0AgSwBaQk8JaCon1LxHAECBAgQGERAUQ8yCDEIECCQJSBtLwFF3UvaPgQIECBA4A4BRX0HmlsIECBAIEsgOa2iTp6e7AQIECAwvYCinn7EDkiAAAECWQLnaRX1uYffCBAgQIDAUAKKeqhxCEOAAAECBM4FRi/q87R+I0CAAAECxQQUdbGBOy4BAgQIZAko6i3nZS0CBAgQILCxgKLeGNRyBAgQIEBgSwFFvaVm1lrSEiBAgECAgKIOGJKIBAgQIFBXQFHXnX3WyaUlQIBAUQFFXXTwjk2AAAECGQKKOmNOUmYJSEuAAIHNBBT1ZpQWIkCAAAEC2wso6u1NrUggS0BaAgSGFlDUQ49HOAIECBCoLqCoq78DnJ9AloC0BMoJKOpyI3dgAgQIEEgSUNRJ05KVAIEsAWkJbCCgqDdAtAQBAgQIEGgloKhbyVqXAAECWQLSDiqgqAcdjFgECBAgQOAkoKhPCh4ECBAgkCVQKK2iLjRsRyVAgACBPAFFnTcziQkQIEAgS2BVWkW9is/NBAgQIECgrYCibutrdQIECBAgsEqge1GvSutmAgQIECBQTEBRFxu44xIgQIBAloCivjgvLxIgQIAAgX0FFPW+/nYnQIAAAQIXBRT1RZ6sF6UlQIAAgfkEFPV8M3UiAgQIEJhIQFFPNMyso0hLgAABArcIKOpblFxDgAABAgR2ElDUO8HbNktAWgIECOwloKj3krcvAQIECBC4QUBR34DkEgJZAtISIDCTgKKeaZrOQoAAAQLTCSjq6UbqQASyBKQlQOCygKK+7ONVAgQIECCwq4Ci3pXf5gQIZAlIS6C/gKLub25HAgQIECBws4CivpnKhQQIEMgSkHYOAUU9xxydggABAgQmFVDUkw7WsQgQIJAlIO1zAor6ORnPEyBAgACBAQQU9QBDEIEAAQIEsgR6plXUPbXtRYAAAQIEFgoo6oVgLidAgAABAj0F1hd1z7T2IkCAAAECxQQUdbGBOy4BAgQIZAlUK+qs6UhLgAABAuUFFHX5twAAAgQIEBhZQFGPPB3ZCBAgQKC8gKIu/xYAQIAAAQIjCyjqkaeTlU1aAgQIEGggoKgboFqSAAECBAhsJfAJAAD//2gk0qUAAAAGSURBVAMA5EUZeFzwojwAAAAASUVORK5CYII=</t>
         </is>
       </c>
-      <c r="CQ5" t="inlineStr"/>
-      <c r="CR5" t="inlineStr"/>
       <c r="CS5" t="inlineStr">
         <is>
           <t>संधारित की जा रही है</t>
         </is>
       </c>
-      <c r="CT5" t="inlineStr"/>
       <c r="CU5" t="inlineStr">
         <is>
           <t>2081</t>
@@ -2763,19 +2769,21 @@
           <t>0</t>
         </is>
       </c>
-      <c r="CX5" t="inlineStr"/>
-      <c r="CY5" t="inlineStr"/>
-      <c r="CZ5" t="inlineStr"/>
       <c r="DA5" t="inlineStr">
         <is>
           <t>0</t>
         </is>
       </c>
-      <c r="DB5" t="inlineStr"/>
-      <c r="DC5" t="inlineStr"/>
-      <c r="DD5" t="inlineStr"/>
-      <c r="DE5" t="inlineStr"/>
-      <c r="DF5" t="inlineStr"/>
+      <c r="DH5" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="DJ5" t="inlineStr">
+        <is>
+          <t>समय पर पेश किये जाते हैं</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -3146,6 +3154,1779 @@
       <c r="DA6" t="inlineStr">
         <is>
           <t>0</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>REP-MOCK-20260609-2212</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>2026-06-09T09:05:40.640138</t>
+        </is>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K7" t="inlineStr">
+        <is>
+          <t>1990-01-01</t>
+        </is>
+      </c>
+      <c r="L7" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="M7" t="inlineStr">
+        <is>
+          <t>स्नातक (Graduate)</t>
+        </is>
+      </c>
+      <c r="N7" t="inlineStr">
+        <is>
+          <t>2015-08-15</t>
+        </is>
+      </c>
+      <c r="O7" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="P7" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="Q7" t="inlineStr">
+        <is>
+          <t>स्थाई</t>
+        </is>
+      </c>
+      <c r="R7" t="inlineStr">
+        <is>
+          <t>प्रशिक्षित</t>
+        </is>
+      </c>
+      <c r="S7" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="T7" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="U7" t="inlineStr">
+        <is>
+          <t>सरकारी पटवार घर</t>
+        </is>
+      </c>
+      <c r="V7" t="inlineStr">
+        <is>
+          <t>तन्हा निवास</t>
+        </is>
+      </c>
+      <c r="W7" t="inlineStr">
+        <is>
+          <t>कोई नोटिस जारी नहीं।</t>
+        </is>
+      </c>
+      <c r="X7" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही विचाराधीन नहीं।</t>
+        </is>
+      </c>
+      <c r="Y7" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही निर्णित नहीं।</t>
+        </is>
+      </c>
+      <c r="Z7" t="inlineStr">
+        <is>
+          <t>निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया।</t>
+        </is>
+      </c>
+      <c r="AA7" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="AB7" t="inlineStr">
+        <is>
+          <t>हस्ताक्षर लिये गये हैं</t>
+        </is>
+      </c>
+      <c r="AC7" t="inlineStr">
+        <is>
+          <t>चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।</t>
+        </is>
+      </c>
+      <c r="AD7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","v_name":"भिनाय","v_khata":"350","v_khasra":"1420","v_area":"482.50","v_lagan":"3200","v_cultivable":"390.00","v_sivaychak":"62.50","v_pasture":"30.00"}]</t>
+        </is>
+      </c>
+      <c r="AK7" t="inlineStr">
+        <is>
+          <t>गत निरीक्षण के निर्देशों की पालना की जा चुकी है।</t>
+        </is>
+      </c>
+      <c r="AL7" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"","ins_officer":"तहसीलदार भिनाय","ins_date":"2025-10-15","ins_receive_date":"2025-10-20","ins_compliance_date":"2025-10-25"}],"remarks":"गत निरीक्षण के निर्देशों की पालना की जा चुकी है।"}</t>
+        </is>
+      </c>
+      <c r="AM7" t="inlineStr">
+        <is>
+          <t>{"diary_pages":"हाँ","diary_blank_pages":"हाँ","diary_certified":"हाँ","diary_period":"हाँ","diary_extraordinary":"लागू नहीं","diary_govt_work":"हाँ","diary_recovery":"हाँ","diary_annual_reg":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="AN7" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","map_jamabandi":"0","map_sheet1":"0","map_sheet2":"0","map_diff_reason":"कोई अन्तर नहीं"}],"remarks":"जमाबंदी व नक्शा खसरा मिलान में कोई महत्वपूर्ण अन्तर नहीं पाया गया।"}</t>
+        </is>
+      </c>
+      <c r="AO7" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","g_samvat":"2082","g_rotation":"","g_crop":"","g_goswara":"अंकित","g_kharaba":"नहीं","g_trees":"नहीं","g_encroach":"नहीं","g_zero":"नहीं"}],"remarks":"निर्धारित प्रपत्र में संधारित की जा रही है/ऑनलाइन की जा रही है"}</t>
+        </is>
+      </c>
+      <c r="AP7" t="inlineStr">
+        <is>
+          <t>["जांच की गई","जांच की गई","इन्द्राज पूर्ण","विवरण अंकित","रिपोर्ट समय पर प्रेषित","पूर्ति की गई"]</t>
+        </is>
+      </c>
+      <c r="AQ7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","e_sivay_count":"0","e_past_count":"0","e_sivay_check":"जांच की गई","e_past_check":"जांच की गई","e_sivay_enc":"0","e_past_enc":"0","e_report_time":"समय पर","e_report_delay":"समय पर"}]</t>
+        </is>
+      </c>
+      <c r="AR7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","p14_count":"0","p14_report":"लागू नहीं","p14_orders":"लागू नहीं","p14_eviction":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="AS7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","r91_status":"हाँ","r91_complete":"पूर्ण","r91_jinswar_detail":"हाँ","r91_remarks":"सुरक्षित"}]</t>
+        </is>
+      </c>
+      <c r="AT7" t="inlineStr">
+        <is>
+          <t>{"भिनाय":{"खरीफ पी-16":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"रबी पी-17":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"जायद रबी पी-18":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"मिलान खसरा पी-19":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"पूरक मिलान खसरा पी-19क":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false}}}</t>
+        </is>
+      </c>
+      <c r="AU7" t="inlineStr">
+        <is>
+          <t>{"village_table":[{"v_sync_name":"भिनाय","mu_filed":"0","mu_decided":"0","mu_pending":"0","mu_decision_sheet":"0","mu_execution":"पूर्ण","mu_period":"लागू नहीं","mu_reason":"लागू नहीं"}],"levels_table":[{"ml_level_name":"पटवारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"एलआरसी (LRC) स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"भू-अभिलेख निरीक्षक स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"राजस्व अधिकारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"पंचायत स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"निषेधाज्ञा से अवशेष","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""}],"types_table":[{"v_sync_name":"","mtype_village":"","mtype_name":"","mtype_doc_status":"","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"शुद्धिपत्र","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"हकतर्कनामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहननामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहनफक","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"बेचान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"दान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"वसीयत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"न्यायालय आदेश","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"स्थगन नोट","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"सहमति विभाजन","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"समर्पण","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"विरासत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"अन्य","mtype_doc_status":"संलग्न है","mtype_remarks":""}],"sec_12_4":{"mut_illegal":"कोई नहीं","mut_duplicate":"कोई नहीं","mut_reference":"कोई नहीं","mut_blank":"कोई नहीं","mut_glmac":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="AV7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","sh_decided":"0","sh_docs":"पूर्ण है","sh_remarks":"पूर्ण"}]</t>
+        </is>
+      </c>
+      <c r="AW7" t="inlineStr">
+        <is>
+          <t>{"tableA":[{"v_sync_name":"भिनाय","db_khata":"0","db_write":"0","db_check":"0","db_tra":"0","db_pending":"0"}],"tableB":[{"v_sync_name":"भिनाय","db_b_khata":"0","db_b_patwari":"0","db_b_ilr":"0","db_b_tra":"0","db_b_officer":"0","db_b_reason":"लागू नहीं"}],"rule107_remarks":"मांग पत्र नियमानुसार तैयार कर भू-अभिलेख निरीक्षक को प्रेषित किया गया है।","pending_cases":[{"v_sync_name":"भिनाय","pc_total_apps":"0","pc_disposed_apps":"0","pc_pending_apps":"0","pc_patwari_pending":"0","pc_tehsildar_pending":"0","pc_30days_pending":"0"}]}</t>
+        </is>
+      </c>
+      <c r="AX7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","rec_head":"भू-राजस्व","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"विविध","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"सिंचाई","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"नहर","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अति0 लगान","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अन्य","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AY7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","tr_head":"भू-राजस्व","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"विविध","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"सिंचाई","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"नहर","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अति0 लगान","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अन्य","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AZ7" t="inlineStr">
+        <is>
+          <t>{"copy_reg_status":"हाँ","copy_total_issued":"150","copy_pending_apps":"0","copy_fee_deposited":"हाँ","copy_serial_order":"हाँ","copy_fee_serial":"101 से 250","copy_fee_amount":"3000","copy_fee_words":"तीन हजार रुपये","copy_monthly_meeting_deposit":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="BA7" t="inlineStr">
+        <is>
+          <t>{"store_reg_status":"हाँ","store_verification_date":"2026-04-10","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37":{"p37_reg_status":"हाँ","p37_unavailable_samvat":"लागू नहीं","p37_submitted_upto":"2080","p37_pending_samvat":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="BB7" t="inlineStr">
+        <is>
+          <t>{"passbook_total_holders":"850","passbook_total_dist":"840","passbook_pending":"10","passbook_completed":"840","passbook_fee_status":"पासबुकों का राजकीय शुल्क जमा करा दिया गया है"}</t>
+        </is>
+      </c>
+      <c r="BC7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","nk_custodian":"0","nk_allottee":"0","nk_settled":"0","nk_leaseholder":"0"}]</t>
+        </is>
+      </c>
+      <c r="BD7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cv_khasra":"कोई नहीं","cv_purpose":"लागू नहीं","cv_action":"लागू नहीं","cv_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BE7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cc_order_date":"लागू नहीं","cc_purpose":"लागू नहीं","cc_actual":"लागू नहीं","cc_action":"लागू नहीं","cc_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BF7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cm_order_date":"लागू नहीं","cm_entry":"लागू नहीं","cm_sale":"लागू नहीं","cm_mutation":"लागू नहीं","cm_others":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BG7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","al_order_date":"लागू नहीं","al_purpose":"लागू नहीं","al_actual":"लागू नहीं","al_action":"लागू नहीं","al_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BH7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","ga_offices":"0","ga_cases":"0","ga_pending":"0","ga_private":"0","ga_diff":"0"}]</t>
+        </is>
+      </c>
+      <c r="BI7" t="inlineStr">
+        <is>
+          <t>{"seeding":[{"v_sync_name":"भिनाय","sd_ver_pending":"0","sd_land":"0","sd_aadhaar":"0"}],"znms":[{"v_sync_name":"भिनाय","zn_draft":"0","zn_ver":"0","zn_znms":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BJ7" t="inlineStr">
+        <is>
+          <t>{"relief":[{"v_sync_name":"भिनाय","di_fire":"0","di_flood":"0","di_house":"0","di_lightning":"0","di_others":"0"}],"accidents":[{"v_sync_name":"भिनाय","ac_accident":"0","ac_drown":"0","ac_elec":"0","ac_collapse":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BK7" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","bs_total":"0","bs_bank":"0","bs_aadhaar":"0","bs_errors":"0"}]</t>
+        </is>
+      </c>
+      <c r="BL7" t="inlineStr">
+        <is>
+          <t>{"rule116_status":"संधारित है","rule116_sign":"हस्ताक्षर लिये गये हैं","rule117_egras":"चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।","copy_reg_status":"हाँ","store_reg_status":"हाँ","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37_reg_status":"हाँ","passbook_total_dist":"840","seeding_remarks":"पीएम किसान योजना के अंतर्गत सीडिंग व फार्मर रजिस्ट्री का कार्य लगभग पूर्ण हो चुका है।","r91_active_count":"1","r91_inactive_count":"0","r91_overall_remarks":"सीमा चिन्ह सुरक्षित अवस्था में हैं तथा सीमांकन रजिस्टर पूर्ण है।","jinswar_remarks":"सामयिक फसल विवरण पत्र (जिंसवार) समय पर प्रस्तुत किए गए हैं।","rule121_pending_date":"","copy_remarks":"नकल पंजिका पूर्ण व अद्यतन है, राजकीय शुल्क समय पर जमा है।","store_remarks":"सर्वे यंत्र पंजिका पूर्ण व अद्यतन है।","passbook_remarks":"कृषि जोत पासबुक का अधिकांश वितरण पूर्ण हो चुका है, शेष प्रगति पर है।","r89_register_status":"संधारित की जा रही है","check_girdawari_remarks":"नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।","dhal_samvat":"2081","dhal_year":"2024","recovery_not_started_count":"0","recovery_last_date":"2026-05-31","recovery_pending_start_date":"2026-04-01","recovery_pending_end_date":"2026-05-31","seamaprakaran_total_pending":"0","seamaprakaran_remarks":"लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।","citizen_charter_register_status":"नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।","grievances_register_status":"अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।","rti_register_status":"सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।","govt_schemes_progress":"राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।","conclusion_text":"निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया। अभिलेखों का संधारण नियमानुसार अद्यतन है।","sdm_dispatch_no":"","sdm_dispatch_date":"","sdm_dispatch_tehsil":"","sdm_dispatch_patwari_circle":"","sdm_dispatch_patwari_tehsil":"","cv_remarks":"कृषि भूमि का विधि विपरीत अकृषि उपयोग का कोई नवीन प्रकरण ध्यान में नहीं आया है।","cc_remarks":"रूपांतरित भूमि का उपयोग स्वीकृत प्रयोजनार्थ ही किया जा रहा है।","al_remarks":"राजकीय प्रयोजनार्थ आवंटित भूमि का उपयोग संबंधित विभागों द्वारा नियमानुसार किया जा रहा है।","ga_remarks":"राजकीय कार्यालयों को आवंटित भूमियों का रिकॉर्ड में नियमानुसार अमल दर्ज है।","court_cases_remarks":"बकाया वसूली प्रकरणों में कुर्की व नीलामी की कार्रवाई प्रगति पर है।","nk_inst_custodian":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_allottee":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_settled":"बंदोबस्त रिकॉर्ड अनुसार खातेदारी अधिकार दिए गए हैं।","nk_inst_leaseholder":"लीज शर्तो की पालना सुनिश्चित की जा रही है।","exam_passed_year":"2015","dhal_remarks":"ढालबांछों का मिलान व प्रमाणीकरण समय पर पूर्ण किया गया है।","recovery_remarks":"राजस्व वसूली नियमित रूप से कर राजकोष में जमा कराई जा रही है।","rule116_remarks":"काश्तकारों को रसीदें प्रदान कर उनके हस्ताक्षर लिए गए हैं।","accidents_remarks":"दुर्घटना/डूबने/विद्युत आपदा राहत के सभी प्रकरणों में समय पर सहायता राशि स्वीकृत कराई गई है।","diary_duty_compliance":"हाँ","diary_duty_remarks":"पालना की जा रही है","jinswar_submit_status":"समय पर पेश किये जाते हैं"}</t>
+        </is>
+      </c>
+      <c r="BM7" t="inlineStr">
+        <is>
+          <t>{"summary":{"mact":"0","lr":"0","pdr":"0","irr":"0","audit":"0"},"cases":[{"type":"MACT","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"LR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"PDR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"IRR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"Audit","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""}]}</t>
+        </is>
+      </c>
+      <c r="BT7" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="BU7" t="inlineStr">
+        <is>
+          <t>{"pending":[{"p_sec_name":"111, 128","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"131","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"136","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"53","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"88","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"251ए","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"188","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"अन्य","p_sec_count":"0","p_sec_period":"0"}],"decided":[{"d_sec_name":"111, 128","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"131","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"136","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"53","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"88","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"251ए","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"188","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"अन्य","d_sec_count":"0","d_sec_period":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BV7" t="inlineStr">
+        <is>
+          <t>[{"v_name":"भिनाय","double_tenant":0,"blank_accounts":0,"adjacent_khasras":0,"no_share":0,"minor_guardian":0,"respectful_caste":0,"no_caste":0,"khatedar_nonkhatedar":0,"govt_pasture_mixed":0,"abadi_cremation_govt":0,"private_mortgage":0,"temple_mafi":0,"path_cremation_only":0,"no_conversion_govt":0,"adopted_son":0,"different_castes":0,"grandson_parentage":0,"deceased_inheritance":0,"conversion_purpose_mismatch":0,"no_separate_account":0,"school_playground_govt":0,"path_surrendered":0,"converted_in_zeroone":0,"other_corrections":0}]</t>
+        </is>
+      </c>
+      <c r="BW7" t="inlineStr">
+        <is>
+          <t>{"circ_1":"पूर्ण","circ_2":"हाँ","circ_3":"हाँ","circ_4":"125 दिनांक 15/05/2026","circ_5":"आदेश पुस्तक अद्यतन है।","circ_status":"बनी हुई है","circ_order_no":"125","circ_order_date":"2026-05-15","circ_order_subject":"राजस्व कार्य समीक्षा","remarks":"आदेश पंजिका में सभी महत्वपूर्ण आदेश अंकित हैं।"}</t>
+        </is>
+      </c>
+      <c r="BX7" t="inlineStr">
+        <is>
+          <t>{"remarks":"कोई विशेष कमी नहीं पाई गई।","status":"समय पर","jan":"2026-01-05","feb":"2026-02-05","mar":"2026-03-05","apr":"2026-04-05","may":"2026-05-05","jun":"2026-06-05","jul":"2026-07-05","aug":"2026-08-05","sep":"2026-09-05","oct":"2026-10-05","nov":"2026-11-05","dec":"2026-12-05"}</t>
+        </is>
+      </c>
+      <c r="BY7" t="inlineStr">
+        <is>
+          <t>नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।</t>
+        </is>
+      </c>
+      <c r="BZ7" t="inlineStr">
+        <is>
+          <t>अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।</t>
+        </is>
+      </c>
+      <c r="CA7" t="inlineStr">
+        <is>
+          <t>सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।</t>
+        </is>
+      </c>
+      <c r="CB7" t="inlineStr">
+        <is>
+          <t>राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।</t>
+        </is>
+      </c>
+      <c r="CC7" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="CD7" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="CS7" t="inlineStr">
+        <is>
+          <t>संधारित की जा रही है</t>
+        </is>
+      </c>
+      <c r="CT7" t="inlineStr">
+        <is>
+          <t>नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।</t>
+        </is>
+      </c>
+      <c r="CU7" t="inlineStr">
+        <is>
+          <t>2081</t>
+        </is>
+      </c>
+      <c r="CV7" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CW7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CX7" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="CY7" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="CZ7" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="DA7" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DB7" t="inlineStr">
+        <is>
+          <t>लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।</t>
+        </is>
+      </c>
+      <c r="DC7" t="inlineStr">
+        <is>
+          <t>निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया। अभिलेखों का संधारण नियमानुसार अद्यतन है।</t>
+        </is>
+      </c>
+      <c r="DG7" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="DH7" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="DI7" t="inlineStr">
+        <is>
+          <t>पालना की जा रही है</t>
+        </is>
+      </c>
+      <c r="DJ7" t="inlineStr">
+        <is>
+          <t>समय पर पेश किये जाते हैं</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>REP-MOCK-20260609-5647</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>2026-06-09T09:11:33.946775</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K8" t="inlineStr">
+        <is>
+          <t>1990-01-01</t>
+        </is>
+      </c>
+      <c r="L8" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="M8" t="inlineStr">
+        <is>
+          <t>स्नातक (Graduate)</t>
+        </is>
+      </c>
+      <c r="N8" t="inlineStr">
+        <is>
+          <t>2015-08-15</t>
+        </is>
+      </c>
+      <c r="O8" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="P8" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="Q8" t="inlineStr">
+        <is>
+          <t>स्थाई</t>
+        </is>
+      </c>
+      <c r="R8" t="inlineStr">
+        <is>
+          <t>प्रशिक्षित</t>
+        </is>
+      </c>
+      <c r="S8" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="T8" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="U8" t="inlineStr">
+        <is>
+          <t>सरकारी पटवार घर</t>
+        </is>
+      </c>
+      <c r="V8" t="inlineStr">
+        <is>
+          <t>तन्हा निवास</t>
+        </is>
+      </c>
+      <c r="W8" t="inlineStr">
+        <is>
+          <t>कोई नोटिस जारी नहीं।</t>
+        </is>
+      </c>
+      <c r="X8" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही विचाराधीन नहीं।</t>
+        </is>
+      </c>
+      <c r="Y8" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही निर्णित नहीं।</t>
+        </is>
+      </c>
+      <c r="Z8" t="inlineStr">
+        <is>
+          <t>निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया।</t>
+        </is>
+      </c>
+      <c r="AA8" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="AB8" t="inlineStr">
+        <is>
+          <t>हस्ताक्षर लिये गये हैं</t>
+        </is>
+      </c>
+      <c r="AC8" t="inlineStr">
+        <is>
+          <t>चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।</t>
+        </is>
+      </c>
+      <c r="AD8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","v_name":"भिनाय","v_khata":"350","v_khasra":"1420","v_area":"482.50","v_lagan":"3200","v_cultivable":"390.00","v_sivaychak":"62.50","v_pasture":"30.00"}]</t>
+        </is>
+      </c>
+      <c r="AK8" t="inlineStr">
+        <is>
+          <t>गत निरीक्षण के निर्देशों की पालना की जा चुकी है।</t>
+        </is>
+      </c>
+      <c r="AL8" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"","ins_officer":"तहसीलदार भिनाय","ins_date":"2025-10-15","ins_receive_date":"2025-10-20","ins_compliance_date":"2025-10-25"}],"remarks":"गत निरीक्षण के निर्देशों की पालना की जा चुकी है।"}</t>
+        </is>
+      </c>
+      <c r="AM8" t="inlineStr">
+        <is>
+          <t>{"diary_pages":"हाँ","diary_blank_pages":"हाँ","diary_certified":"हाँ","diary_period":"हाँ","diary_extraordinary":"लागू नहीं","diary_govt_work":"हाँ","diary_recovery":"हाँ","diary_annual_reg":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="AN8" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","map_jamabandi":"0","map_sheet1":"0","map_sheet2":"0","map_diff_reason":"कोई अन्तर नहीं"}],"remarks":"जमाबंदी व नक्शा खसरा मिलान में कोई महत्वपूर्ण अन्तर नहीं पाया गया।"}</t>
+        </is>
+      </c>
+      <c r="AO8" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","g_samvat":"2082","g_rotation":"","g_crop":"","g_goswara":"अंकित","g_kharaba":"नहीं","g_trees":"नहीं","g_encroach":"नहीं","g_zero":"नहीं"}],"remarks":"निर्धारित प्रपत्र में संधारित की जा रही है/ऑनलाइन की जा रही है"}</t>
+        </is>
+      </c>
+      <c r="AP8" t="inlineStr">
+        <is>
+          <t>["जांच की गई","जांच की गई","इन्द्राज पूर्ण","विवरण अंकित","रिपोर्ट समय पर प्रेषित","पूर्ति की गई"]</t>
+        </is>
+      </c>
+      <c r="AQ8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","e_sivay_count":"0","e_past_count":"0","e_sivay_check":"जांच की गई","e_past_check":"जांच की गई","e_sivay_enc":"0","e_past_enc":"0","e_report_time":"समय पर","e_report_delay":"समय पर"}]</t>
+        </is>
+      </c>
+      <c r="AR8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","p14_count":"0","p14_report":"लागू नहीं","p14_orders":"लागू नहीं","p14_eviction":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="AS8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","r91_status":"हाँ","r91_complete":"पूर्ण","r91_jinswar_detail":"हाँ","r91_remarks":"सुरक्षित"}]</t>
+        </is>
+      </c>
+      <c r="AT8" t="inlineStr">
+        <is>
+          <t>{"भिनाय":{"खरीफ पी-16":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"रबी पी-17":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"जायद रबी पी-18":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"मिलान खसरा पी-19":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"पूरक मिलान खसरा पी-19क":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false}}}</t>
+        </is>
+      </c>
+      <c r="AU8" t="inlineStr">
+        <is>
+          <t>{"village_table":[{"v_sync_name":"भिनाय","mu_filed":"0","mu_decided":"0","mu_pending":"0","mu_decision_sheet":"0","mu_execution":"पूर्ण","mu_period":"लागू नहीं","mu_reason":"लागू नहीं"}],"levels_table":[{"ml_level_name":"पटवारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"एलआरसी (LRC) स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"भू-अभिलेख निरीक्षक स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"राजस्व अधिकारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"पंचायत स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"निषेधाज्ञा से अवशेष","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""}],"types_table":[{"v_sync_name":"","mtype_village":"","mtype_name":"","mtype_doc_status":"","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"शुद्धिपत्र","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"हकतर्कनामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहननामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहनफक","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"बेचान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"दान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"वसीयत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"न्यायालय आदेश","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"स्थगन नोट","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"सहमति विभाजन","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"समर्पण","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"विरासत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"अन्य","mtype_doc_status":"संलग्न है","mtype_remarks":""}],"sec_12_4":{"mut_illegal":"कोई नहीं","mut_duplicate":"कोई नहीं","mut_reference":"कोई नहीं","mut_blank":"कोई नहीं","mut_glmac":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="AV8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","sh_decided":"0","sh_docs":"पूर्ण है","sh_remarks":"पूर्ण"}]</t>
+        </is>
+      </c>
+      <c r="AW8" t="inlineStr">
+        <is>
+          <t>{"tableA":[{"v_sync_name":"भिनाय","db_khata":"0","db_write":"0","db_check":"0","db_tra":"0","db_pending":"0"}],"tableB":[{"v_sync_name":"भिनाय","db_b_khata":"0","db_b_patwari":"0","db_b_ilr":"0","db_b_tra":"0","db_b_officer":"0","db_b_reason":"लागू नहीं"}],"rule107_remarks":"मांग पत्र नियमानुसार तैयार कर भू-अभिलेख निरीक्षक को प्रेषित किया गया है।","pending_cases":[{"v_sync_name":"भिनाय","pc_total_apps":"0","pc_disposed_apps":"0","pc_pending_apps":"0","pc_patwari_pending":"0","pc_tehsildar_pending":"0","pc_30days_pending":"0"}]}</t>
+        </is>
+      </c>
+      <c r="AX8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","rec_head":"भू-राजस्व","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"विविध","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"सिंचाई","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"नहर","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अति0 लगान","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अन्य","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AY8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","tr_head":"भू-राजस्व","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"विविध","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"सिंचाई","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"नहर","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अति0 लगान","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अन्य","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AZ8" t="inlineStr">
+        <is>
+          <t>{"copy_reg_status":"हाँ","copy_total_issued":"150","copy_pending_apps":"0","copy_fee_deposited":"हाँ","copy_serial_order":"हाँ","copy_fee_serial":"101 से 250","copy_fee_amount":"3000","copy_fee_words":"तीन हजार रुपये","copy_monthly_meeting_deposit":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="BA8" t="inlineStr">
+        <is>
+          <t>{"store_reg_status":"हाँ","store_verification_date":"2026-04-10","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37":{"p37_reg_status":"हाँ","p37_unavailable_samvat":"लागू नहीं","p37_submitted_upto":"2080","p37_pending_samvat":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="BB8" t="inlineStr">
+        <is>
+          <t>{"passbook_total_holders":"850","passbook_total_dist":"840","passbook_pending":"10","passbook_completed":"840","passbook_fee_status":"पासबुकों का राजकीय शुल्क जमा करा दिया गया है"}</t>
+        </is>
+      </c>
+      <c r="BC8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","nk_custodian":"0","nk_allottee":"0","nk_settled":"0","nk_leaseholder":"0"}]</t>
+        </is>
+      </c>
+      <c r="BD8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cv_khasra":"कोई नहीं","cv_purpose":"लागू नहीं","cv_action":"लागू नहीं","cv_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BE8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cc_order_date":"लागू नहीं","cc_purpose":"लागू नहीं","cc_actual":"लागू नहीं","cc_action":"लागू नहीं","cc_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BF8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cm_order_date":"लागू नहीं","cm_entry":"लागू नहीं","cm_sale":"लागू नहीं","cm_mutation":"लागू नहीं","cm_others":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BG8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","al_order_date":"लागू नहीं","al_purpose":"लागू नहीं","al_actual":"लागू नहीं","al_action":"लागू नहीं","al_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BH8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","ga_offices":"0","ga_cases":"0","ga_pending":"0","ga_private":"0","ga_diff":"0"}]</t>
+        </is>
+      </c>
+      <c r="BI8" t="inlineStr">
+        <is>
+          <t>{"seeding":[{"v_sync_name":"भिनाय","sd_ver_pending":"0","sd_land":"0","sd_aadhaar":"0"}],"znms":[{"v_sync_name":"भिनाय","zn_draft":"0","zn_ver":"0","zn_znms":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BJ8" t="inlineStr">
+        <is>
+          <t>{"relief":[{"v_sync_name":"भिनाय","di_fire":"0","di_flood":"0","di_house":"0","di_lightning":"0","di_others":"0"}],"accidents":[{"v_sync_name":"भिनाय","ac_accident":"0","ac_drown":"0","ac_elec":"0","ac_collapse":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BK8" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","bs_total":"0","bs_bank":"0","bs_aadhaar":"0","bs_errors":"0"}]</t>
+        </is>
+      </c>
+      <c r="BL8" t="inlineStr">
+        <is>
+          <t>{"rule116_status":"संधारित है","rule116_sign":"हस्ताक्षर लिये गये हैं","rule117_egras":"चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।","copy_reg_status":"हाँ","store_reg_status":"हाँ","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37_reg_status":"हाँ","passbook_total_dist":"840","seeding_remarks":"पीएम किसान योजना के अंतर्गत सीडिंग व फार्मर रजिस्ट्री का कार्य लगभग पूर्ण हो चुका है।","r91_active_count":"1","r91_inactive_count":"0","r91_overall_remarks":"सीमा चिन्ह सुरक्षित अवस्था में हैं तथा सीमांकन रजिस्टर पूर्ण है।","jinswar_remarks":"सामयिक फसल विवरण पत्र (जिंसवार) समय पर प्रस्तुत किए गए हैं।","rule121_pending_date":"","copy_remarks":"नकल पंजिका पूर्ण व अद्यतन है, राजकीय शुल्क समय पर जमा है।","store_remarks":"सर्वे यंत्र पंजिका पूर्ण व अद्यतन है।","passbook_remarks":"कृषि जोत पासबुक का अधिकांश वितरण पूर्ण हो चुका है, शेष प्रगति पर है।","r89_register_status":"संधारित की जा रही है","check_girdawari_remarks":"नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।","dhal_samvat":"2081","dhal_year":"2024","recovery_not_started_count":"0","recovery_last_date":"2026-05-31","recovery_pending_start_date":"2026-04-01","recovery_pending_end_date":"2026-05-31","seamaprakaran_total_pending":"0","seamaprakaran_remarks":"लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।","citizen_charter_register_status":"नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।","grievances_register_status":"अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।","rti_register_status":"सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।","govt_schemes_progress":"राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।","conclusion_text":"निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया। अभिलेखों का संधारण नियमानुसार अद्यतन है।","sdm_dispatch_no":"","sdm_dispatch_date":"","sdm_dispatch_tehsil":"","sdm_dispatch_patwari_circle":"","sdm_dispatch_patwari_tehsil":"","cv_remarks":"कृषि भूमि का विधि विपरीत अकृषि उपयोग का कोई नवीन प्रकरण ध्यान में नहीं आया है।","cc_remarks":"रूपांतरित भूमि का उपयोग स्वीकृत प्रयोजनार्थ ही किया जा रहा है।","al_remarks":"राजकीय प्रयोजनार्थ आवंटित भूमि का उपयोग संबंधित विभागों द्वारा नियमानुसार किया जा रहा है।","ga_remarks":"राजकीय कार्यालयों को आवंटित भूमियों का रिकॉर्ड में नियमानुसार अमल दर्ज है।","court_cases_remarks":"बकाया वसूली प्रकरणों में कुर्की व नीलामी की कार्रवाई प्रगति पर है।","nk_inst_custodian":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_allottee":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_settled":"बंदोबस्त रिकॉर्ड अनुसार खातेदारी अधिकार दिए गए हैं।","nk_inst_leaseholder":"लीज शर्तो की पालना सुनिश्चित की जा रही है।","exam_passed_year":"2015","dhal_remarks":"ढालबांछों का मिलान व प्रमाणीकरण समय पर पूर्ण किया गया है।","recovery_remarks":"राजस्व वसूली नियमित रूप से कर राजकोष में जमा कराई जा रही है।","rule116_remarks":"काश्तकारों को रसीदें प्रदान कर उनके हस्ताक्षर लिए गए हैं।","accidents_remarks":"दुर्घटना/डूबने/विद्युत आपदा राहत के सभी प्रकरणों में समय पर सहायता राशि स्वीकृत कराई गई है।","diary_duty_compliance":"हाँ","diary_duty_remarks":"पालना की जा रही है","jinswar_submit_status":"समय पर पेश किये जाते हैं"}</t>
+        </is>
+      </c>
+      <c r="BM8" t="inlineStr">
+        <is>
+          <t>{"summary":{"mact":"0","lr":"0","pdr":"0","irr":"0","audit":"0"},"cases":[{"type":"MACT","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"LR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"PDR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"IRR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"Audit","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""}]}</t>
+        </is>
+      </c>
+      <c r="BT8" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="BU8" t="inlineStr">
+        <is>
+          <t>{"pending":[{"p_sec_name":"111, 128","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"131","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"136","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"53","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"88","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"251ए","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"188","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"अन्य","p_sec_count":"0","p_sec_period":"0"}],"decided":[{"d_sec_name":"111, 128","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"131","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"136","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"53","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"88","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"251ए","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"188","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"अन्य","d_sec_count":"0","d_sec_period":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BV8" t="inlineStr">
+        <is>
+          <t>[{"v_name":"भिनाय","double_tenant":0,"blank_accounts":0,"adjacent_khasras":0,"no_share":0,"minor_guardian":0,"respectful_caste":0,"no_caste":0,"khatedar_nonkhatedar":0,"govt_pasture_mixed":0,"abadi_cremation_govt":0,"private_mortgage":0,"temple_mafi":0,"path_cremation_only":0,"no_conversion_govt":0,"adopted_son":0,"different_castes":0,"grandson_parentage":0,"deceased_inheritance":0,"conversion_purpose_mismatch":0,"no_separate_account":0,"school_playground_govt":0,"path_surrendered":0,"converted_in_zeroone":0,"other_corrections":0}]</t>
+        </is>
+      </c>
+      <c r="BW8" t="inlineStr">
+        <is>
+          <t>{"circ_1":"पूर्ण","circ_2":"हाँ","circ_3":"हाँ","circ_4":"125 दिनांक 15/05/2026","circ_5":"आदेश पुस्तक अद्यतन है।","circ_status":"बनी हुई है","circ_order_no":"125","circ_order_date":"2026-05-15","circ_order_subject":"राजस्व कार्य समीक्षा","remarks":"आदेश पंजिका में सभी महत्वपूर्ण आदेश अंकित हैं।"}</t>
+        </is>
+      </c>
+      <c r="BX8" t="inlineStr">
+        <is>
+          <t>{"remarks":"कोई विशेष कमी नहीं पाई गई।","status":"समय पर","jan":"2026-01-05","feb":"2026-02-05","mar":"2026-03-05","apr":"2026-04-05","may":"2026-05-05","jun":"2026-06-05","jul":"2026-07-05","aug":"2026-08-05","sep":"2026-09-05","oct":"2026-10-05","nov":"2026-11-05","dec":"2026-12-05"}</t>
+        </is>
+      </c>
+      <c r="BY8" t="inlineStr">
+        <is>
+          <t>नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।</t>
+        </is>
+      </c>
+      <c r="BZ8" t="inlineStr">
+        <is>
+          <t>अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।</t>
+        </is>
+      </c>
+      <c r="CA8" t="inlineStr">
+        <is>
+          <t>सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।</t>
+        </is>
+      </c>
+      <c r="CB8" t="inlineStr">
+        <is>
+          <t>राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।</t>
+        </is>
+      </c>
+      <c r="CC8" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="CD8" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="CS8" t="inlineStr">
+        <is>
+          <t>संधारित की जा रही है</t>
+        </is>
+      </c>
+      <c r="CT8" t="inlineStr">
+        <is>
+          <t>नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।</t>
+        </is>
+      </c>
+      <c r="CU8" t="inlineStr">
+        <is>
+          <t>2081</t>
+        </is>
+      </c>
+      <c r="CV8" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CW8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CX8" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="CY8" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="CZ8" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="DA8" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DB8" t="inlineStr">
+        <is>
+          <t>लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।</t>
+        </is>
+      </c>
+      <c r="DC8" t="inlineStr">
+        <is>
+          <t>निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया। अभिलेखों का संधारण नियमानुसार अद्यतन है।</t>
+        </is>
+      </c>
+      <c r="DG8" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="DH8" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="DI8" t="inlineStr">
+        <is>
+          <t>पालना की जा रही है</t>
+        </is>
+      </c>
+      <c r="DJ8" t="inlineStr">
+        <is>
+          <t>समय पर पेश किये जाते हैं</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>REP-MOCK-20260609-3046</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>2026-06-09T09:13:59.539738</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K9" t="inlineStr">
+        <is>
+          <t>1990-01-01</t>
+        </is>
+      </c>
+      <c r="L9" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="M9" t="inlineStr">
+        <is>
+          <t>स्नातक (Graduate)</t>
+        </is>
+      </c>
+      <c r="N9" t="inlineStr">
+        <is>
+          <t>2015-08-15</t>
+        </is>
+      </c>
+      <c r="O9" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="P9" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="Q9" t="inlineStr">
+        <is>
+          <t>स्थाई</t>
+        </is>
+      </c>
+      <c r="R9" t="inlineStr">
+        <is>
+          <t>प्रशिक्षित</t>
+        </is>
+      </c>
+      <c r="S9" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="T9" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="U9" t="inlineStr">
+        <is>
+          <t>सरकारी पटवार घर</t>
+        </is>
+      </c>
+      <c r="V9" t="inlineStr">
+        <is>
+          <t>तन्हा निवास</t>
+        </is>
+      </c>
+      <c r="W9" t="inlineStr">
+        <is>
+          <t>कोई नोटिस जारी नहीं।</t>
+        </is>
+      </c>
+      <c r="X9" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही विचाराधीन नहीं।</t>
+        </is>
+      </c>
+      <c r="Y9" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही निर्णित नहीं।</t>
+        </is>
+      </c>
+      <c r="Z9" t="inlineStr">
+        <is>
+          <t>निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया।</t>
+        </is>
+      </c>
+      <c r="AA9" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="AB9" t="inlineStr">
+        <is>
+          <t>हस्ताक्षर लिये गये हैं</t>
+        </is>
+      </c>
+      <c r="AC9" t="inlineStr">
+        <is>
+          <t>चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।</t>
+        </is>
+      </c>
+      <c r="AD9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","v_name":"भिनाय","v_khata":"350","v_khasra":"1420","v_area":"482.50","v_lagan":"3200","v_cultivable":"390.00","v_sivaychak":"62.50","v_pasture":"30.00"}]</t>
+        </is>
+      </c>
+      <c r="AK9" t="inlineStr">
+        <is>
+          <t>गत निरीक्षण के निर्देशों की पालना की जा चुकी है।</t>
+        </is>
+      </c>
+      <c r="AL9" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"","ins_officer":"तहसीलदार भिनाय","ins_date":"2025-10-15","ins_receive_date":"2025-10-20","ins_compliance_date":"2025-10-25"}],"remarks":"गत निरीक्षण के निर्देशों की पालना की जा चुकी है।"}</t>
+        </is>
+      </c>
+      <c r="AM9" t="inlineStr">
+        <is>
+          <t>{"diary_pages":"हाँ","diary_blank_pages":"हाँ","diary_certified":"हाँ","diary_period":"हाँ","diary_extraordinary":"लागू नहीं","diary_govt_work":"हाँ","diary_recovery":"हाँ","diary_annual_reg":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="AN9" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","map_jamabandi":"0","map_sheet1":"0","map_sheet2":"0","map_diff_reason":"कोई अन्तर नहीं"}],"remarks":"जमाबंदी व नक्शा खसरा मिलान में कोई महत्वपूर्ण अन्तर नहीं पाया गया।"}</t>
+        </is>
+      </c>
+      <c r="AO9" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","g_samvat":"2082","g_rotation":"","g_crop":"","g_goswara":"अंकित","g_kharaba":"नहीं","g_trees":"नहीं","g_encroach":"नहीं","g_zero":"नहीं"}],"remarks":"निर्धारित प्रपत्र में संधारित की जा रही है/ऑनलाइन की जा रही है"}</t>
+        </is>
+      </c>
+      <c r="AP9" t="inlineStr">
+        <is>
+          <t>["जांच की गई","जांच की गई","इन्द्राज पूर्ण","विवरण अंकित","रिपोर्ट समय पर प्रेषित","पूर्ति की गई"]</t>
+        </is>
+      </c>
+      <c r="AQ9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","e_sivay_count":"0","e_past_count":"0","e_sivay_check":"जांच की गई","e_past_check":"जांच की गई","e_sivay_enc":"0","e_past_enc":"0","e_report_time":"समय पर","e_report_delay":"समय पर"}]</t>
+        </is>
+      </c>
+      <c r="AR9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","p14_count":"0","p14_report":"लागू नहीं","p14_orders":"लागू नहीं","p14_eviction":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="AS9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","r91_status":"हाँ","r91_complete":"पूर्ण","r91_jinswar_detail":"हाँ","r91_remarks":"सुरक्षित"}]</t>
+        </is>
+      </c>
+      <c r="AT9" t="inlineStr">
+        <is>
+          <t>{"भिनाय":{"खरीफ पी-16":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"रबी पी-17":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"जायद रबी पी-18":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"मिलान खसरा पी-19":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"पूरक मिलान खसरा पी-19क":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false}}}</t>
+        </is>
+      </c>
+      <c r="AU9" t="inlineStr">
+        <is>
+          <t>{"village_table":[{"v_sync_name":"भिनाय","mu_filed":"0","mu_decided":"0","mu_pending":"0","mu_decision_sheet":"0","mu_execution":"पूर्ण","mu_period":"लागू नहीं","mu_reason":"लागू नहीं"}],"levels_table":[{"ml_level_name":"पटवारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"एलआरसी (LRC) स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"भू-अभिलेख निरीक्षक स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"राजस्व अधिकारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"पंचायत स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"निषेधाज्ञा से अवशेष","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""}],"types_table":[{"v_sync_name":"","mtype_village":"","mtype_name":"","mtype_doc_status":"","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"शुद्धिपत्र","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"हकतर्कनामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहननामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहनफक","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"बेचान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"दान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"वसीयत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"न्यायालय आदेश","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"स्थगन नोट","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"सहमति विभाजन","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"समर्पण","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"विरासत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"अन्य","mtype_doc_status":"संलग्न है","mtype_remarks":""}],"sec_12_4":{"mut_illegal":"कोई नहीं","mut_duplicate":"कोई नहीं","mut_reference":"कोई नहीं","mut_blank":"कोई नहीं","mut_glmac":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="AV9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","sh_decided":"0","sh_docs":"पूर्ण है","sh_remarks":"पूर्ण"}]</t>
+        </is>
+      </c>
+      <c r="AW9" t="inlineStr">
+        <is>
+          <t>{"tableA":[{"v_sync_name":"भिनाय","db_khata":"0","db_write":"0","db_check":"0","db_tra":"0","db_pending":"0"}],"tableB":[{"v_sync_name":"भिनाय","db_b_khata":"0","db_b_patwari":"0","db_b_ilr":"0","db_b_tra":"0","db_b_officer":"0","db_b_reason":"लागू नहीं"}],"rule107_remarks":"मांग पत्र नियमानुसार तैयार कर भू-अभिलेख निरीक्षक को प्रेषित किया गया है।","pending_cases":[{"v_sync_name":"भिनाय","pc_total_apps":"0","pc_disposed_apps":"0","pc_pending_apps":"0","pc_patwari_pending":"0","pc_tehsildar_pending":"0","pc_30days_pending":"0"}]}</t>
+        </is>
+      </c>
+      <c r="AX9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","rec_head":"भू-राजस्व","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"विविध","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"सिंचाई","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"नहर","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अति0 लगान","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अन्य","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AY9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","tr_head":"भू-राजस्व","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"विविध","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"सिंचाई","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"नहर","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अति0 लगान","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अन्य","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AZ9" t="inlineStr">
+        <is>
+          <t>{"copy_reg_status":"हाँ","copy_total_issued":"150","copy_pending_apps":"0","copy_fee_deposited":"हाँ","copy_serial_order":"हाँ","copy_fee_serial":"101 से 250","copy_fee_amount":"3000","copy_fee_words":"तीन हजार रुपये","copy_monthly_meeting_deposit":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="BA9" t="inlineStr">
+        <is>
+          <t>{"store_reg_status":"हाँ","store_verification_date":"2026-04-10","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37":{"p37_reg_status":"हाँ","p37_unavailable_samvat":"लागू नहीं","p37_submitted_upto":"2080","p37_pending_samvat":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="BB9" t="inlineStr">
+        <is>
+          <t>{"passbook_total_holders":"850","passbook_total_dist":"840","passbook_pending":"10","passbook_completed":"840","passbook_fee_status":"पासबुकों का राजकीय शुल्क जमा करा दिया गया है"}</t>
+        </is>
+      </c>
+      <c r="BC9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","nk_custodian":"0","nk_allottee":"0","nk_settled":"0","nk_leaseholder":"0"}]</t>
+        </is>
+      </c>
+      <c r="BD9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cv_khasra":"कोई नहीं","cv_purpose":"लागू नहीं","cv_action":"लागू नहीं","cv_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BE9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cc_order_date":"लागू नहीं","cc_purpose":"लागू नहीं","cc_actual":"लागू नहीं","cc_action":"लागू नहीं","cc_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BF9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cm_order_date":"लागू नहीं","cm_entry":"लागू नहीं","cm_sale":"लागू नहीं","cm_mutation":"लागू नहीं","cm_others":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BG9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","al_order_date":"लागू नहीं","al_purpose":"लागू नहीं","al_actual":"लागू नहीं","al_action":"लागू नहीं","al_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BH9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","ga_offices":"0","ga_cases":"0","ga_pending":"0","ga_private":"0","ga_diff":"0"}]</t>
+        </is>
+      </c>
+      <c r="BI9" t="inlineStr">
+        <is>
+          <t>{"seeding":[{"v_sync_name":"भिनाय","sd_ver_pending":"0","sd_land":"0","sd_aadhaar":"0"}],"znms":[{"v_sync_name":"भिनाय","zn_draft":"0","zn_ver":"0","zn_znms":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BJ9" t="inlineStr">
+        <is>
+          <t>{"relief":[{"v_sync_name":"भिनाय","di_fire":"0","di_flood":"0","di_house":"0","di_lightning":"0","di_others":"0"}],"accidents":[{"v_sync_name":"भिनाय","ac_accident":"0","ac_drown":"0","ac_elec":"0","ac_collapse":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BK9" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","bs_total":"0","bs_bank":"0","bs_aadhaar":"0","bs_errors":"0"}]</t>
+        </is>
+      </c>
+      <c r="BL9" t="inlineStr">
+        <is>
+          <t>{"rule116_status":"संधारित है","rule116_sign":"हस्ताक्षर लिये गये हैं","rule117_egras":"चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।","copy_reg_status":"हाँ","store_reg_status":"हाँ","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37_reg_status":"हाँ","passbook_total_dist":"840","seeding_remarks":"पीएम किसान योजना के अंतर्गत सीडिंग व फार्मर रजिस्ट्री का कार्य लगभग पूर्ण हो चुका है।","r91_active_count":"1","r91_inactive_count":"0","r91_overall_remarks":"सीमा चिन्ह सुरक्षित अवस्था में हैं तथा सीमांकन रजिस्टर पूर्ण है।","jinswar_remarks":"सामयिक फसल विवरण पत्र (जिंसवार) समय पर प्रस्तुत किए गए हैं।","rule121_pending_date":"","copy_remarks":"नकल पंजिका पूर्ण व अद्यतन है, राजकीय शुल्क समय पर जमा है।","store_remarks":"सर्वे यंत्र पंजिका पूर्ण व अद्यतन है।","passbook_remarks":"कृषि जोत पासबुक का अधिकांश वितरण पूर्ण हो चुका है, शेष प्रगति पर है।","r89_register_status":"संधारित की जा रही है","check_girdawari_remarks":"नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।","dhal_samvat":"2081","dhal_year":"2024","recovery_not_started_count":"0","recovery_last_date":"2026-05-31","recovery_pending_start_date":"2026-04-01","recovery_pending_end_date":"2026-05-31","seamaprakaran_total_pending":"0","seamaprakaran_remarks":"लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।","citizen_charter_register_status":"नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।","grievances_register_status":"अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।","rti_register_status":"सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।","govt_schemes_progress":"राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।","conclusion_text":"निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया। अभिलेखों का संधारण नियमानुसार अद्यतन है।","sdm_dispatch_no":"","sdm_dispatch_date":"","sdm_dispatch_tehsil":"","sdm_dispatch_patwari_circle":"","sdm_dispatch_patwari_tehsil":"","cv_remarks":"कृषि भूमि का विधि विपरीत अकृषि उपयोग का कोई नवीन प्रकरण ध्यान में नहीं आया है।","cc_remarks":"रूपांतरित भूमि का उपयोग स्वीकृत प्रयोजनार्थ ही किया जा रहा है।","al_remarks":"राजकीय प्रयोजनार्थ आवंटित भूमि का उपयोग संबंधित विभागों द्वारा नियमानुसार किया जा रहा है।","ga_remarks":"राजकीय कार्यालयों को आवंटित भूमियों का रिकॉर्ड में नियमानुसार अमल दर्ज है।","court_cases_remarks":"बकाया वसूली प्रकरणों में कुर्की व नीलामी की कार्रवाई प्रगति पर है।","nk_inst_custodian":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_allottee":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_settled":"बंदोबस्त रिकॉर्ड अनुसार खातेदारी अधिकार दिए गए हैं।","nk_inst_leaseholder":"लीज शर्तो की पालना सुनिश्चित की जा रही है।","exam_passed_year":"2015","dhal_remarks":"ढालबांछों का मिलान व प्रमाणीकरण समय पर पूर्ण किया गया है।","recovery_remarks":"राजस्व वसूली नियमित रूप से कर राजकोष में जमा कराई जा रही है।","rule116_remarks":"काश्तकारों को रसीदें प्रदान कर उनके हस्ताक्षर लिए गए हैं।","accidents_remarks":"दुर्घटना/डूबने/विद्युत आपदा राहत के सभी प्रकरणों में समय पर सहायता राशि स्वीकृत कराई गई है।","diary_duty_compliance":"हाँ","diary_duty_remarks":"पालना की जा रही है","jinswar_submit_status":"समय पर पेश किये जाते हैं"}</t>
+        </is>
+      </c>
+      <c r="BM9" t="inlineStr">
+        <is>
+          <t>{"summary":{"mact":"0","lr":"0","pdr":"0","irr":"0","audit":"0"},"cases":[{"type":"MACT","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"LR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"PDR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"IRR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"Audit","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""}]}</t>
+        </is>
+      </c>
+      <c r="BN9" t="inlineStr">
+        <is>
+          <t>data:image/png;base64,iVBORw0KGgoAAAANSUhEUgAAAfEAAACVCAYAAABIIMOFAAAQAElEQVR4AezdC5Bb1X3H8f+R1sY2Xkk2u7rCOBMeO4AkB8Y41IEwaRIIEMqrTVMKJAylkNIMBAIMTUlIpmmBMKGhQCktCUlpGkI6tE2ghDA80xSSUN5YWoe64CbG1l3DWld+QGyvTv9X0nrwg80+JN2Hvpp7dB+S7jnnc7z723uvJCeEGwIIIIAAAghEUoAQj+Sw0WgEEEAAAQREgglx5BFAAAEEEEBgxgKE+IwJ2QECCCCAAALBCPRSiAcjTK0IIIAAAgh0SIAQ7xAsu0UAAQQQQKDTAoR4p4XZPwIIIIAAAh0SIMQ7BMtuEUAAAQQQ6LQAId5p4WD2T60IIIAAAj0gQIj3wCDTRQQQQACBeAoQ4vEc12B6Ra0IIIAAAl0VIMS7yk1lCCCAAAIItE+AEG+fJXsKRoBaEUAAgZ4VIMR7dujpOAIIIIBA1AUI8aiPIO0PRoBaEUAAgRAIEOIhGASagAACCCCAwHQECPHpqPEaBIIRoFYEEEBgJwFCfCcOVhBAAAEEEIiOACEenbGipQgEI0CtCCAQWgFCPLRDQ8MQQAABBBCYWIAQn9iHRxFAIBgBakUAgUkIEOKTQOIpCCCAAAIIhFGAEA/jqNAmBBAIRoBaEYiYACEesQGjuQgggAACCIwLEOLjEswRQACBYASoFYFpCxDi06bjhQgggAACCAQrQIgH60/tCCCAQDAC1BoLAUI8FsNIJxBAAAEEelGAEO/FUafPCCCAQDAC1NpmAUK8zaDsDgEEEEAAgW4JEOLdkqYeBBBAAIFgBGJcKyEe48GlawgggAAC8RYgxOM9vvQOAQQQQCAYga7USoh3hZlKEEAAAQQQaL8AId5+U/aIAAIIIIBAVwR2C/Gu1EolCCCAAAIIIDBjAUJ8xoTsAAEEEEAAgWAEQhLiwXSeWhFAAAEEEIiyACEe5dGj7QgggAACPS3Q0yHe0yNP5xFAAAEEIi9AiEd+COkAAggggECvChDiXR95KkQAAQQQQKA9AoR4exzZCwIIIIAAAl0XIMS7Th5MhdSKAAIIIBA/AUI8fmNKjxBAAAEEekSAEO+RgQ6mm9SKAAIIINBJAUK8k7rsGwEEEEAAgQ4KEOIdxGXXwQhQKwIIINArAoR4r4w0/UQAAQQQiJ0AIR67IaVDwQhQKwIIINB9AUK8++bUiAACCCCAQFsECPG2MLITBIIRoFYEEOhtAUK8t8ef3iOAAAIIRFiAEI/w4NF0BDovsP+chdlDj9q5HtYQQCAsAoR4WEaCdiAQJoGhob3STuGqtDNv45hJPNk/WDg3TM2jLQgg0BQgxJsO3COAgC+w//5zUrniF9MbZ6/W1Wu09GmRRFKW+PMgC3UjgMDuAoT47iZsQaAnBeYN5PfNvDlvvbH2LxQgp2V8WuVVyleMrzBHAIHwCBDi4RkLWoJAYAKZbPHwvqR52orMbzbCjDTnem/s7XrfoxPdRiDcAoR4uMeH1iHQcYF+Z8nJ1tgnjcgirawuYu8Wa47W5cZkrOzXWOAOAQRCJ0CIh25IaBAC3RPIZAuXJ6T+A61xnpZN1pqTPHfeOWLG7tb1xmSN9DcWuOuaABUhMFkBQnyyUjwPgXgJJFO54p0a0Ddot/zfA6+NGbO8NlJ6MOO8+U0R815p3lZ6leFPNRe5RwCBsAn4P7xhaxPtQQCBDgosWHBgOu0UHjLWntOoxsoz221i2aZKqZzO5a/U6+KfaGwX82py29blujymhSn2AnQwigKEeBRHjTYjME2BtPOeA+t7zXlKX/4hLSLG/ps3b8sxm0dWuKls8QSx5ivSvNXqY2Mnjo6uqjVXuUcAgTAKEOJhHBXahEAHBBYMFo4RGXtarBzs796I+Ss9Vf4xWb36rfm5YsEYe49uNyJGz6yb0ze+vvJl4YZAhwXY/cwECPGZ+fFqBCIhkMnmz6kn5FFt7AItW63YM6tu6Wpdlvm5ocGktT/S5cbHy/Q6+SXVSukxXWdCAIGQCxDiIR8gmofATAX0+ve11pg7dT+ztLyu17w/UHOHW+8+XzYraWffr9vfpUUn841apXSrLjAhEGOB+HSNEI/PWNITBHYWWLx4bjpX8I+w/7zxgJGXE0lZVnPLP2+s613znehypC7602OeW7rQX6AggEA0BAjxaIwTrURgSgLpgfwR6W0pV6yc0HrhI8mtW4/csLb8y9a67OGd6KfrY7wTXRGYEOiEQCf2SYh3QpV9IhCgQNrJny9J89/ahNaXtNinPbd8wtvfac470VWHCYEYCBDiMRhEuoCALzA4WJifyeX/ScR8XURaP9v2e5477J8u33GEPT9XKBpj/1WfY0R4J7pwQyDCAq0f9Al6wEMIIBB+gUJh9takrLfWfLLVWFcT+nQN8D9srTdmAwOHLOqz1j9K37uxwdYv5p3oDQnuEIikACEeyWGj0QjsLJB5XS7W699zGluNPJfc1vfeqlv2vxO9scm/S+WKR25LJl+wYub662LM497I8G2NZe4QQCCSAmEN8UhihqXRCxcOpcLSFtrRBQE9CrdGrmjVtNmbs+Xo0dEX17TWG7NUNv9JY+0TujKgxZ+e9yq/PtFfoCCAQHQFCPHojt0eW552lvx0bNZsL5XL/84en8DG2AmkX5fztFM5LWKsfMn/BjZ/uVUS6VzhBmOMXisX/3Pidd1+leeWl4qs+rUuMyGAQIQFCPG3D17Elx3nML3OWX+f3w39ZT5+bdRfpcRVQI/CxWhwN/v3RnXelh1f1LJQz8ikncKDYuXy5sOyyRp7igb4da11ZgggEHEBQjziA/j25m+q11ofKfK3mjP8r9r0lyjxFdjlKPy68aPw1GBxSM/IPKM9P06LP62uJ5NH1irDP/RXKAggEA8BQjz4cWxbCzavX13RAb1qfIfWmDtTg4WLxteZx1DAyI2tXlXHj8LTTv44k7B+gA+1Hvux7JU8YuPal1a21pkhgEBMBPR3fkx6QjcaAhvc8nVGzGmNFb0zCbkllSv8tS4yxUygeflEmu9IF1tduG3O0nS2cIWIeVBEGm9utGJu0tPnx3q/fGmDbmNCAIGYCRDiMRtQvztVt3SvsYnf85f9YqxclnKKesT2wT5/vVG4i7zApvr2t18+2X9se+JJvT7+Ve2Y/3O91Rg5r+aWLtX1HV/0ostMCCAQIwH/hz1G3aEr4wLVkRX/LnW5yoo03oFsxF6acUYe33uw0HgX8/jzmEdXYPP6csUkzNVWzMhuvbByr7Vjj++2nQ0IIBArAUI8VsO5c2e89f6p9bG8bh3WIlbk/X0JebE/u+Rofz2AQpVtEkg5+felncJ3bN1+Uf9Ay+62WyO/L5J8JeMUbkk7hxyw2+NsQACBWAgQ4rEYxnfuhOf+4tX+WbVl+oy7tPjTYMLUf5zJFsY/duRvo0RBYGhoLw3l8/S69zNGzE+1yWdp8T/7LWLtS0bkW5K0H9E/1nZ8U5suXyQa5mkn/0o6W7w17RQvyAwWls4byO/rfwRNX8+EAAIRFiDEIzx4k236mjVr3vTc8tli5U/1NVu19FkjN6Scwg9ab47STTGeIt61hYuWvEsD+Pr0xtmvaSjfode9j2h1abPO/2HMmKI3MnxY1S2f560dfrjmlk83Cfvb+twdYS5iDhBjP61pf7tNyLOzkmbtGF8KJNwQiLoAIR71EZxC+72R8t+buvhfBvOa/zIjcupbsv2F/uyhnF73QUJW0tklx+sfWveOjdVXawBfqc3bR4toiL+sp9AvTW7bukj/OLtwU6VUll1u1XXD/+mHeSIpF+tDT2l5Xst2LbtO7951A+sIIBAdAUI8OmPVlpZW15efq/fVD9edPaLFnw5KmMQTaSf/UH+2+H5/A6UtAtPaycDAIf0pp/CZdK7wCzH1B/UPrVN0R/7PaV2PrO+z1pzoVcqHVt3hm0ZHV9X0sQmnDWvLf6tBv1zLUm8f2VvPwCw3CfM3dSP3SEL+pFYZ/rsJd8CDCCAQagH/l0OoG0jj2i+w8bWVb+gv9eN1z9dqaU3muISx/5XOFp5pfNOb/3WerUeYdV6gf9Ehh2hw37YtmVyrwX2TXvo4uFXrqFjzVT09fqAeWZ9aGyn5nwHXPG89OpVZuby1Vik/VV1X+uzGSvnj3rry7VN5Oc9FAIHwCRDi4RuTbrWorkH+eWsT5+h1Uv9NUm81KjZyhDXmzvQbsibtFK7hI2kNlU7dJdPZ4sfSTv6xxFhypVi5UCuar0WHRJ7VMP9jb+6W/byR0pV6evz/Gtt/0x2PI4BATwkQ4j013Lt3tjay4tueO3y0Xl91jJjL9BmvaPGnQb27qi8hv0o7xbv5WJpqtGHq3+/QffSI+w8yTuGf005hixh7j4j5oDRv/jXrf6lbc4w3Ul5WdcvflNWrm39cNR/nHgEEENhJgBDfiaN3V/zrq1W3dKPnlocSYk4VMQ9J89anh4VnJEz9iXS28HQmmz9HONXelJnMvVppWB+bzhavT6tfYnvidT3i/p6eDz9bXz5bi4iRUb3W/aXtNrFY/c/YOFLy/99vidCNpiKAQEACiYDqpdrwCtgNbuk+zy0db+v2YDHmNm2q/1EmESPLWqfaf5Vxin/JqXbZ422Bk1+ScYqf1SPuB/SyhKdPeliPuK/0/XR5fHreGnunrnzeq2Sd2kjpy5tHVri6zoQAAghMWoAQnzRV7z2xtn74f7xK6dN6qn2RHjl+RsS8Ks1b1or9gp5qX5fJFn6SyhY+sXDhUOM/3Gg+3Fv3/inylFM8Ux2+pUfda+piXlKfr+kR94kq0foPSuQ1a+UfrZiz6n31AT3iXlqrDJ+r82tFHvdPo+tTmaYkwJMRQEAIcf4R/EaB0dFVtZpbvkWPzg/So8eT9QUPa2lM1sgxxsi3x2bNfkMD7H4NsvgHeuMUefHDaSf/FT3aflZPka83Yu9Sh3MVZT8t/rRFQ/wBI+aypJElGtaLayPlP6q5pe/6nw7wn0BBAAEEZipAiM9UsLdeb/Xo8X4NpI8kEts/oF3/voh9Uef+pNfO5SQNMj/QPQ24LRrqFS2rdPkFnT+p5aGUU/i+zr+TdvK3p5zijZlc/su6/rmUU7g44xTOSzv5M/qdJSdncsUPpXKF35qfKxYy++bf3b/o4IHFixfPnZ8bGgyi7OMUlmf8U+TZwg/1FPkG7fcjIubPNKiXiuiJct2g98/p7HpdPdbbRxZ4I+WTqm7pxtFKuSTc4iJAPxAIlQAhHqrhiE5jNqx7+SeeW/5dzx0+XGxiSMPrC1rGA107YubqnaPlIBFzmIgcpeU4I3Kazs8SMRfo0eul1pqrReQ63X6zFblDxNydkPp91tpHjZWfJ60t2bpZnRjrW79xW2pL0s4eCaLo+e6fNU6RG/moiMzT4k96DdvcYcWcrafIB71K+Qj1+JyesXhUymX/623951AQQACBjgkQ4h2j7Z0deyMr/lfD6xoth+vp9ZM0nP/DitwsYr6hwf5dXb5XRPTIVX6m4IpyugAABCNJREFU85e0+B9j8//7TP8Nc/qwbonApH9wbNOj7R8ZPUWeEPsezy3nNLDP11Pkd3GKPAIDGOUm0nYE3kGAEH8HGDZPT6BWKT9QdYdP0Wvol3hu6QLPHT5Ll0/z3PJxWo7ScpiWg7Q4WuZrSeydnLv3mNmaNaZ+gH/92BpZboz5cELMqXr0e6b+IXC+Jv0lOv+6/3WhJmEus8Zc1MXyNaN/lNQG7Hw92v5oVU+Rb3CHV0xPiFchgAAC7RNItG9X7AmB6QmsXfvMlk2VVeurlZWr/evH+ofAU9VK6TH/o241d/huzx2+o+aWb9b5pzZWyh+vrivdWKuUbu1iubzqli/hFPn0xpdXRVaAhkdAgBCPwCDRRAQQQAABBPYkQIjvSYVtCCCAAALBCFDrlAQI8Slx8WQEEEAAAQTCI0CIh2csaAkCCCCAQDACka2VEI/s0NFwBBBAAIFeFyDEe/1fAP1HAAEEEAhGoA21EuJtQGQXCCCAAAIIBCFAiAehTp0IIIAAAgi0QWAaId6GWtkFAggggAACCMxYgBCfMSE7QAABBBBAIBiByIR4MDzUigACCCCAQHgFCPHwjg0tQwABBBBAYEIBQnxCHh5EAAEEEEAgvAKEeHjHhpYhgAACCCAwoQAhPiFPMA9SKwIIIIAAApMRIMQno8RzEEAAAQQQCKEAIR7CQQmmSdSKAAIIIBA1AUI8aiNGexFAAAEEEGgJEOItCGbBCFArAggggMD0BQjx6dvxSgQQQAABBAIVIMQD5afyYASoFQEEEIiHACEej3GkFwgggAACPShAiPfgoNPlYASoFQEEEGi3ACHeblH2hwACCCCAQJcECPEuQVMNAsEIUCsCCMRZgBCP8+jSNwQQQACBWAsQ4rEeXjqHQDAC1IoAAt0RIMS740wtCCCAAAIItF2AEG87KTtEAIFgBKgVgd4TIMR7b8zpMQIIIIBATAQI8ZgMJN1AAIFgBKgVgSAFCPEg9akbAQQQQACBGQgQ4jPA46UIIIBAMALUikBTgBBvOnCPAAIIIIBA5AQI8cgNGQ1GAAEEghGg1vAJEOLhGxNahAACCCCAwKQECPFJMfEkBBBAAIFgBKh1IgFCfCIdHkMAAQQQQCDEAoR4iAeHpiGAAAIIBCMQlVoJ8aiMFO1EAAEEEEBgFwFCfBcQVhFAAAEEEAhGYOq1EuJTN+MVCCCAAAIIhEKAEA/FMNAIBBBAAAEEpi7QjhCfeq28AgEEEEAAAQRmLECIz5iQHSCAAAIIIBCMQHRDPBgvakUAAQQQQCA0AoR4aIaChiCAAAIIIDA1AUJ8al48GwEEEEAAgdAIEOKhGQoaggACCCCAwNQECPGpeQXzbGpFAAEEEEBgDwKE+B5Q2IQAAggggEAUBAjxKIxSMG2kVgQQQACBkAv8PwAAAP//WknFeQAAAAZJREFUAwAP6AN227t96gAAAABJRU5ErkJggg==</t>
+        </is>
+      </c>
+      <c r="BT9" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="BU9" t="inlineStr">
+        <is>
+          <t>{"pending":[{"p_sec_name":"111, 128","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"131","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"136","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"53","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"88","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"251ए","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"188","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"अन्य","p_sec_count":"0","p_sec_period":"0"}],"decided":[{"d_sec_name":"111, 128","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"131","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"136","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"53","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"88","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"251ए","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"188","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"अन्य","d_sec_count":"0","d_sec_period":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BV9" t="inlineStr">
+        <is>
+          <t>[{"v_name":"भिनाय","double_tenant":0,"blank_accounts":0,"adjacent_khasras":0,"no_share":0,"minor_guardian":0,"respectful_caste":0,"no_caste":0,"khatedar_nonkhatedar":0,"govt_pasture_mixed":0,"abadi_cremation_govt":0,"private_mortgage":0,"temple_mafi":0,"path_cremation_only":0,"no_conversion_govt":0,"adopted_son":0,"different_castes":0,"grandson_parentage":0,"deceased_inheritance":0,"conversion_purpose_mismatch":0,"no_separate_account":0,"school_playground_govt":0,"path_surrendered":0,"converted_in_zeroone":0,"other_corrections":0}]</t>
+        </is>
+      </c>
+      <c r="BW9" t="inlineStr">
+        <is>
+          <t>{"circ_1":"पूर्ण","circ_2":"हाँ","circ_3":"हाँ","circ_4":"125 दिनांक 15/05/2026","circ_5":"आदेश पुस्तक अद्यतन है।","circ_status":"बनी हुई है","circ_order_no":"125","circ_order_date":"2026-05-15","circ_order_subject":"राजस्व कार्य समीक्षा","remarks":"आदेश पंजिका में सभी महत्वपूर्ण आदेश अंकित हैं।"}</t>
+        </is>
+      </c>
+      <c r="BX9" t="inlineStr">
+        <is>
+          <t>{"remarks":"कोई विशेष कमी नहीं पाई गई।","status":"समय पर","jan":"2026-01-05","feb":"2026-02-05","mar":"2026-03-05","apr":"2026-04-05","may":"2026-05-05","jun":"2026-06-05","jul":"2026-07-05","aug":"2026-08-05","sep":"2026-09-05","oct":"2026-10-05","nov":"2026-11-05","dec":"2026-12-05"}</t>
+        </is>
+      </c>
+      <c r="BY9" t="inlineStr">
+        <is>
+          <t>नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।</t>
+        </is>
+      </c>
+      <c r="BZ9" t="inlineStr">
+        <is>
+          <t>अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।</t>
+        </is>
+      </c>
+      <c r="CA9" t="inlineStr">
+        <is>
+          <t>सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।</t>
+        </is>
+      </c>
+      <c r="CB9" t="inlineStr">
+        <is>
+          <t>राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।</t>
+        </is>
+      </c>
+      <c r="CC9" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="CD9" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="CS9" t="inlineStr">
+        <is>
+          <t>संधारित की जा रही है</t>
+        </is>
+      </c>
+      <c r="CT9" t="inlineStr">
+        <is>
+          <t>नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।</t>
+        </is>
+      </c>
+      <c r="CU9" t="inlineStr">
+        <is>
+          <t>2081</t>
+        </is>
+      </c>
+      <c r="CV9" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CW9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CX9" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="CY9" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="CZ9" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="DA9" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DB9" t="inlineStr">
+        <is>
+          <t>लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।</t>
+        </is>
+      </c>
+      <c r="DC9" t="inlineStr">
+        <is>
+          <t>निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया। अभिलेखों का संधारण नियमानुसार अद्यतन है।</t>
+        </is>
+      </c>
+      <c r="DG9" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="DH9" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="DI9" t="inlineStr">
+        <is>
+          <t>पालना की जा रही है</t>
+        </is>
+      </c>
+      <c r="DJ9" t="inlineStr">
+        <is>
+          <t>समय पर पेश किये जाते हैं</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>REP-MOCK-20260609-2684</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>2026-06-09T09:43:24.753199</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr"/>
+      <c r="D10" t="inlineStr"/>
+      <c r="E10" t="inlineStr"/>
+      <c r="F10" t="inlineStr"/>
+      <c r="G10" t="inlineStr"/>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t>1990-01-01</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t>स्नातक (Graduate)</t>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t>2015-08-15</t>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="P10" t="inlineStr">
+        <is>
+          <t>35000</t>
+        </is>
+      </c>
+      <c r="Q10" t="inlineStr">
+        <is>
+          <t>स्थाई</t>
+        </is>
+      </c>
+      <c r="R10" t="inlineStr">
+        <is>
+          <t>प्रशिक्षित</t>
+        </is>
+      </c>
+      <c r="S10" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="T10" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="U10" t="inlineStr">
+        <is>
+          <t>सरकारी पटवार घर</t>
+        </is>
+      </c>
+      <c r="V10" t="inlineStr">
+        <is>
+          <t>तन्हा निवास</t>
+        </is>
+      </c>
+      <c r="W10" t="inlineStr">
+        <is>
+          <t>कोई नोटिस जारी नहीं।</t>
+        </is>
+      </c>
+      <c r="X10" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही विचाराधीन नहीं।</t>
+        </is>
+      </c>
+      <c r="Y10" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही निर्णित नहीं।</t>
+        </is>
+      </c>
+      <c r="Z10" t="inlineStr">
+        <is>
+          <t>निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया।</t>
+        </is>
+      </c>
+      <c r="AA10" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="AB10" t="inlineStr">
+        <is>
+          <t>हस्ताक्षर लिये गये हैं</t>
+        </is>
+      </c>
+      <c r="AC10" t="inlineStr">
+        <is>
+          <t>चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।</t>
+        </is>
+      </c>
+      <c r="AD10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","v_name":"भिनाय","v_khata":"350","v_khasra":"1420","v_area":"482.50","v_lagan":"3200","v_cultivable":"390.00","v_sivaychak":"62.50","v_pasture":"30.00"}]</t>
+        </is>
+      </c>
+      <c r="AK10" t="inlineStr">
+        <is>
+          <t>गत निरीक्षण के निर्देशों की पालना की जा चुकी है।</t>
+        </is>
+      </c>
+      <c r="AL10" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"","ins_officer":"तहसीलदार भिनाय","ins_date":"2025-10-15","ins_receive_date":"2025-10-20","ins_compliance_date":"2025-10-25"}],"remarks":"गत निरीक्षण के निर्देशों की पालना की जा चुकी है।"}</t>
+        </is>
+      </c>
+      <c r="AM10" t="inlineStr">
+        <is>
+          <t>{"diary_pages":"हाँ","diary_blank_pages":"हाँ","diary_certified":"हाँ","diary_period":"हाँ","diary_extraordinary":"लागू नहीं","diary_govt_work":"हाँ","diary_recovery":"हाँ","diary_annual_reg":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="AN10" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","map_jamabandi":"0","map_sheet1":"0","map_sheet2":"0","map_diff_reason":"कोई अन्तर नहीं"}],"remarks":"जमाबंदी व नक्शा खसरा मिलान में कोई महत्वपूर्ण अन्तर नहीं पाया गया।"}</t>
+        </is>
+      </c>
+      <c r="AO10" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","g_samvat":"2082","g_rotation":"","g_crop":"","g_goswara":"अंकित","g_kharaba":"नहीं","g_trees":"नहीं","g_encroach":"नहीं","g_zero":"नहीं"}],"remarks":"निर्धारित प्रपत्र में संधारित की जा रही है/ऑनलाइन की जा रही है"}</t>
+        </is>
+      </c>
+      <c r="AP10" t="inlineStr">
+        <is>
+          <t>["जांच की गई","जांच की गई","इन्द्राज पूर्ण","विवरण अंकित","रिपोर्ट समय पर प्रेषित","पूर्ति की गई"]</t>
+        </is>
+      </c>
+      <c r="AQ10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","e_sivay_count":"0","e_past_count":"0","e_sivay_check":"जांच की गई","e_past_check":"जांच की गई","e_sivay_enc":"0","e_past_enc":"0","e_report_time":"समय पर","e_report_delay":"समय पर"}]</t>
+        </is>
+      </c>
+      <c r="AR10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","p14_count":"0","p14_report":"लागू नहीं","p14_orders":"लागू नहीं","p14_eviction":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="AS10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","r91_status":"हाँ","r91_complete":"पूर्ण","r91_jinswar_detail":"हाँ","r91_remarks":"सुरक्षित"}]</t>
+        </is>
+      </c>
+      <c r="AT10" t="inlineStr">
+        <is>
+          <t>{"भिनाय":{"खरीफ पी-16":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"रबी पी-17":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"जायद रबी पी-18":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"मिलान खसरा पी-19":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"पूरक मिलान खसरा पी-19क":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false}}}</t>
+        </is>
+      </c>
+      <c r="AU10" t="inlineStr">
+        <is>
+          <t>{"village_table":[{"v_sync_name":"भिनाय","mu_filed":"0","mu_decided":"0","mu_pending":"0","mu_decision_sheet":"0","mu_execution":"पूर्ण","mu_period":"लागू नहीं","mu_reason":"लागू नहीं"}],"levels_table":[{"ml_level_name":"पटवारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"एलआरसी (LRC) स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"भू-अभिलेख निरीक्षक स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"राजस्व अधिकारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"पंचायत स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"निषेधाज्ञा से अवशेष","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""}],"types_table":[{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"शुद्धिपत्र","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"हकतर्कनामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहननामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहनफक","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"बेचान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"दान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"वसीयत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"न्यायालय आदेश","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"स्थगन नोट","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"सहमति विभाजन","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"समर्पण","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"विरासत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"अन्य","mtype_doc_status":"संलग्न है","mtype_remarks":""}],"sec_12_4":{"mut_illegal":"कोई नहीं","mut_duplicate":"कोई नहीं","mut_reference":"कोई नहीं","mut_blank":"कोई नहीं","mut_glmac":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="AV10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","sh_decided":"0","sh_docs":"पूर्ण है","sh_remarks":"पूर्ण"}]</t>
+        </is>
+      </c>
+      <c r="AW10" t="inlineStr">
+        <is>
+          <t>{"tableA":[{"v_sync_name":"भिनाय","db_khata":"0","db_write":"0","db_check":"0","db_tra":"0","db_pending":"0"}],"tableB":[{"v_sync_name":"भिनाय","db_b_khata":"0","db_b_patwari":"0","db_b_ilr":"0","db_b_tra":"0","db_b_officer":"0","db_b_reason":"लागू नहीं"}],"rule107_remarks":"मांग पत्र नियमानुसार तैयार कर भू-अभिलेख निरीक्षक को प्रेषित किया गया है।","pending_cases":[{"v_sync_name":"भिनाय","pc_total_apps":"0","pc_disposed_apps":"0","pc_pending_apps":"0","pc_patwari_pending":"0","pc_tehsildar_pending":"0","pc_30days_pending":"0"}]}</t>
+        </is>
+      </c>
+      <c r="AX10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","rec_head":"भू-राजस्व","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"विविध","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"सिंचाई","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"नहर","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अति0 लगान","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अन्य","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AY10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","tr_head":"भू-राजस्व","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"विविध","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"सिंचाई","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"नहर","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अति0 लगान","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अन्य","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AZ10" t="inlineStr">
+        <is>
+          <t>{"copy_reg_status":"हाँ","copy_total_issued":"150","copy_pending_apps":"0","copy_fee_deposited":"हाँ","copy_serial_order":"हाँ","copy_fee_serial":"101 से 250","copy_fee_amount":"3000","copy_fee_words":"तीन हजार रुपये","copy_monthly_meeting_deposit":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="BA10" t="inlineStr">
+        <is>
+          <t>{"store_reg_status":"हाँ","store_verification_date":"2026-04-10","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37":{"p37_reg_status":"हाँ","p37_unavailable_samvat":"लागू नहीं","p37_submitted_upto":"2080","p37_pending_samvat":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="BB10" t="inlineStr">
+        <is>
+          <t>{"passbook_total_holders":"850","passbook_total_dist":"840","passbook_pending":"10","passbook_completed":"840","passbook_fee_status":"पासबुकों का राजकीय शुल्क जमा करा दिया गया है"}</t>
+        </is>
+      </c>
+      <c r="BC10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","nk_custodian":"0","nk_allottee":"0","nk_settled":"0","nk_leaseholder":"0"}]</t>
+        </is>
+      </c>
+      <c r="BD10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cv_khasra":"कोई नहीं","cv_purpose":"लागू नहीं","cv_action":"लागू नहीं","cv_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BE10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cc_order_date":"लागू नहीं","cc_purpose":"लागू नहीं","cc_actual":"लागू नहीं","cc_action":"लागू नहीं","cc_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BF10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cm_order_date":"लागू नहीं","cm_entry":"लागू नहीं","cm_sale":"लागू नहीं","cm_mutation":"लागू नहीं","cm_others":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BG10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","al_order_date":"लागू नहीं","al_purpose":"लागू नहीं","al_actual":"लागू नहीं","al_action":"लागू नहीं","al_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BH10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","ga_offices":"0","ga_cases":"0","ga_pending":"0","ga_private":"0","ga_diff":"0"}]</t>
+        </is>
+      </c>
+      <c r="BI10" t="inlineStr">
+        <is>
+          <t>{"seeding":[{"v_sync_name":"भिनाय","sd_ver_pending":"0","sd_land":"0","sd_aadhaar":"0"}],"znms":[{"v_sync_name":"भिनाय","zn_draft":"0","zn_ver":"0","zn_znms":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BJ10" t="inlineStr">
+        <is>
+          <t>{"relief":[{"v_sync_name":"भिनाय","di_fire":"0","di_flood":"0","di_house":"0","di_lightning":"0","di_others":"0"}],"accidents":[{"v_sync_name":"भिनाय","ac_accident":"0","ac_drown":"0","ac_elec":"0","ac_collapse":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BK10" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","bs_total":"0","bs_bank":"0","bs_aadhaar":"0","bs_errors":"0"}]</t>
+        </is>
+      </c>
+      <c r="BL10" t="inlineStr">
+        <is>
+          <t>{"rule116_status":"संधारित है","rule116_sign":"हस्ताक्षर लिये गये हैं","rule117_egras":"चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।","copy_reg_status":"हाँ","store_reg_status":"हाँ","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37_reg_status":"हाँ","passbook_total_dist":"840","seeding_remarks":"पीएम किसान योजना के अंतर्गत सीडिंग व फार्मर रजिस्ट्री का कार्य लगभग पूर्ण हो चुका है।","r91_active_count":"1","r91_inactive_count":"0","r91_overall_remarks":"सीमा चिन्ह सुरक्षित अवस्था में हैं तथा सीमांकन रजिस्टर पूर्ण है।","jinswar_remarks":"सामयिक फसल विवरण पत्र (जिंसवार) समय पर प्रस्तुत किए गए हैं।","rule121_pending_date":"","copy_remarks":"नकल पंजिका पूर्ण व अद्यतन है, राजकीय शुल्क समय पर जमा है।","store_remarks":"सर्वे यंत्र पंजिका पूर्ण व अद्यतन है।","passbook_remarks":"कृषि जोत पासबुक का अधिकांश वितरण पूर्ण हो चुका है, शेष प्रगति पर है।","r89_register_status":"संधारित की जा रही है","check_girdawari_remarks":"नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।","dhal_samvat":"2081","dhal_year":"2024","recovery_not_started_count":"0","recovery_last_date":"2026-05-31","recovery_pending_start_date":"2026-04-01","recovery_pending_end_date":"2026-05-31","seamaprakaran_total_pending":"0","seamaprakaran_remarks":"लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।","citizen_charter_register_status":"नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।","grievances_register_status":"अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।","rti_register_status":"सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।","govt_schemes_progress":"राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।","conclusion_text":"निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया। अभिलेखों का संधारण नियमानुसार अद्यतन है।","sdm_dispatch_no":"","sdm_dispatch_date":"","sdm_dispatch_tehsil":"","sdm_dispatch_patwari_circle":"","sdm_dispatch_patwari_tehsil":"","cv_remarks":"कृषि भूमि का विधि विपरीत अकृषि उपयोग का कोई नवीन प्रकरण ध्यान में नहीं आया है।","cc_remarks":"रूपांतरित भूमि का उपयोग स्वीकृत प्रयोजनार्थ ही किया जा रहा है।","al_remarks":"राजकीय प्रयोजनार्थ आवंटित भूमि का उपयोग संबंधित विभागों द्वारा नियमानुसार किया जा रहा है।","ga_remarks":"राजकीय कार्यालयों को आवंटित भूमियों का रिकॉर्ड में नियमानुसार अमल दर्ज है।","court_cases_remarks":"बकाया वसूली प्रकरणों में कुर्की व नीलामी की कार्रवाई प्रगति पर है।","nk_inst_custodian":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_allottee":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_settled":"बंदोबस्त रिकॉर्ड अनुसार खातेदारी अधिकार दिए गए हैं।","nk_inst_leaseholder":"लीज शर्तो की पालना सुनिश्चित की जा रही है।","exam_passed_year":"2015","dhal_remarks":"ढालबांछों का मिलान व प्रमाणीकरण समय पर पूर्ण किया गया है।","recovery_remarks":"राजस्व वसूली नियमित रूप से कर राजकोष में जमा कराई जा रही है।","rule116_remarks":"काश्तकारों को रसीदें प्रदान कर उनके हस्ताक्षर लिए गए हैं।","accidents_remarks":"दुर्घटना/डूबने/विद्युत आपदा राहत के सभी प्रकरणों में समय पर सहायता राशि स्वीकृत कराई गई है।","diary_duty_compliance":"हाँ","diary_duty_remarks":"पालना की जा रही है","jinswar_submit_status":"समय पर पेश किये जाते हैं"}</t>
+        </is>
+      </c>
+      <c r="BM10" t="inlineStr">
+        <is>
+          <t>{"summary":{"mact":"0","lr":"0","pdr":"0","irr":"0","audit":"0"},"cases":[{"type":"MACT","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"LR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"PDR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"IRR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"Audit","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""}]}</t>
+        </is>
+      </c>
+      <c r="BO10" t="inlineStr"/>
+      <c r="BP10" t="inlineStr"/>
+      <c r="BQ10" t="inlineStr"/>
+      <c r="BR10" t="inlineStr"/>
+      <c r="BS10" t="inlineStr"/>
+      <c r="BT10" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="BU10" t="inlineStr">
+        <is>
+          <t>{"pending":[{"p_sec_name":"111, 128","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"131","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"136","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"53","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"88","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"251ए","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"188","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"अन्य","p_sec_count":"0","p_sec_period":"0"}],"decided":[{"d_sec_name":"111, 128","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"131","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"136","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"53","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"88","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"251ए","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"188","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"अन्य","d_sec_count":"0","d_sec_period":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BV10" t="inlineStr">
+        <is>
+          <t>[{"v_name":"भिनाय","double_tenant":0,"blank_accounts":0,"adjacent_khasras":0,"no_share":0,"minor_guardian":0,"respectful_caste":0,"no_caste":0,"khatedar_nonkhatedar":0,"govt_pasture_mixed":0,"abadi_cremation_govt":0,"private_mortgage":0,"temple_mafi":0,"path_cremation_only":0,"no_conversion_govt":0,"adopted_son":0,"different_castes":0,"grandson_parentage":0,"deceased_inheritance":0,"conversion_purpose_mismatch":0,"no_separate_account":0,"school_playground_govt":0,"path_surrendered":0,"converted_in_zeroone":0,"other_corrections":0}]</t>
+        </is>
+      </c>
+      <c r="BW10" t="inlineStr">
+        <is>
+          <t>{"circ_1":"पूर्ण","circ_2":"हाँ","circ_3":"हाँ","circ_4":"125 दिनांक 15/05/2026","circ_5":"आदेश पुस्तक अद्यतन है।","circ_status":"बनी हुई है","circ_order_no":"125","circ_order_date":"2026-05-15","circ_order_subject":"राजस्व कार्य समीक्षा","remarks":"आदेश पंजिका में सभी महत्वपूर्ण आदेश अंकित हैं।"}</t>
+        </is>
+      </c>
+      <c r="BX10" t="inlineStr">
+        <is>
+          <t>{"remarks":"कोई विशेष कमी नहीं पाई गई।","status":"समय पर","jan":"2026-01-05","feb":"2026-02-05","mar":"2026-03-05","apr":"2026-04-05","may":"2026-05-05","jun":"2026-06-05","jul":"2026-07-05","aug":"2026-08-05","sep":"2026-09-05","oct":"2026-10-05","nov":"2026-11-05","dec":"2026-12-05"}</t>
+        </is>
+      </c>
+      <c r="BY10" t="inlineStr">
+        <is>
+          <t>नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।</t>
+        </is>
+      </c>
+      <c r="BZ10" t="inlineStr">
+        <is>
+          <t>अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।</t>
+        </is>
+      </c>
+      <c r="CA10" t="inlineStr">
+        <is>
+          <t>सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।</t>
+        </is>
+      </c>
+      <c r="CB10" t="inlineStr">
+        <is>
+          <t>राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।</t>
+        </is>
+      </c>
+      <c r="CC10" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="CD10" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="CQ10" t="inlineStr"/>
+      <c r="CR10" t="inlineStr"/>
+      <c r="CS10" t="inlineStr">
+        <is>
+          <t>संधारित की जा रही है</t>
+        </is>
+      </c>
+      <c r="CT10" t="inlineStr">
+        <is>
+          <t>नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।</t>
+        </is>
+      </c>
+      <c r="CU10" t="inlineStr">
+        <is>
+          <t>2081</t>
+        </is>
+      </c>
+      <c r="CV10" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CW10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CX10" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="CY10" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="CZ10" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="DA10" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DB10" t="inlineStr">
+        <is>
+          <t>लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।</t>
+        </is>
+      </c>
+      <c r="DC10" t="inlineStr">
+        <is>
+          <t>निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया। अभिलेखों का संधारण नियमानुसार अद्यतन है।</t>
+        </is>
+      </c>
+      <c r="DD10" t="inlineStr"/>
+      <c r="DE10" t="inlineStr"/>
+      <c r="DF10" t="inlineStr"/>
+      <c r="DG10" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="DH10" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="DI10" t="inlineStr">
+        <is>
+          <t>पालना की जा रही है</t>
+        </is>
+      </c>
+      <c r="DJ10" t="inlineStr">
+        <is>
+          <t>समय पर पेश किये जाते हैं</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement dynamic dropdown mapping, village selector modal, required fields validation, and SDM auto-save
</commit_message>
<xml_diff>
--- a/patwari_reports.xlsx
+++ b/patwari_reports.xlsx
@@ -717,7 +717,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DJ10"/>
+  <dimension ref="A1:DJ13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <sheetData>
     <row r="1">
@@ -4494,11 +4494,6 @@
           <t>2026-06-09T09:43:24.753199</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>भिनाय</t>
@@ -4789,11 +4784,6 @@
           <t>{"summary":{"mact":"0","lr":"0","pdr":"0","irr":"0","audit":"0"},"cases":[{"type":"MACT","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"LR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"PDR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"IRR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"Audit","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""}]}</t>
         </is>
       </c>
-      <c r="BO10" t="inlineStr"/>
-      <c r="BP10" t="inlineStr"/>
-      <c r="BQ10" t="inlineStr"/>
-      <c r="BR10" t="inlineStr"/>
-      <c r="BS10" t="inlineStr"/>
       <c r="BT10" t="inlineStr">
         <is>
           <t>Pending</t>
@@ -4849,8 +4839,6 @@
           <t>2026-06-01</t>
         </is>
       </c>
-      <c r="CQ10" t="inlineStr"/>
-      <c r="CR10" t="inlineStr"/>
       <c r="CS10" t="inlineStr">
         <is>
           <t>संधारित की जा रही है</t>
@@ -4906,9 +4894,6 @@
           <t>निरीक्षण के दौरान पटवार हल्का का कार्य संतोषजनक पाया गया। अभिलेखों का संधारण नियमानुसार अद्यतन है।</t>
         </is>
       </c>
-      <c r="DD10" t="inlineStr"/>
-      <c r="DE10" t="inlineStr"/>
-      <c r="DF10" t="inlineStr"/>
       <c r="DG10" t="inlineStr">
         <is>
           <t>2015</t>
@@ -4925,6 +4910,1303 @@
         </is>
       </c>
       <c r="DJ10" t="inlineStr">
+        <is>
+          <t>समय पर पेश किये जाते हैं</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>REP-MOCK-20260610-2426</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>2026-06-10T21:49:37.843924</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>उपखंड अधिकारी भिनाय</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t>1990-01-01</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t>स्नातक (Graduate)</t>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t>2015-08-15</t>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="P11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q11" t="inlineStr">
+        <is>
+          <t>स्थाई</t>
+        </is>
+      </c>
+      <c r="R11" t="inlineStr">
+        <is>
+          <t>प्रशिक्षित</t>
+        </is>
+      </c>
+      <c r="S11" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="T11" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="U11" t="inlineStr">
+        <is>
+          <t>सरकारी पटवार घर</t>
+        </is>
+      </c>
+      <c r="V11" t="inlineStr">
+        <is>
+          <t>तन्हा निवास</t>
+        </is>
+      </c>
+      <c r="W11" t="inlineStr">
+        <is>
+          <t>कोई नोटिस जारी नहीं।</t>
+        </is>
+      </c>
+      <c r="X11" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही विचाराधीन नहीं।</t>
+        </is>
+      </c>
+      <c r="Y11" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही निर्णित नहीं।</t>
+        </is>
+      </c>
+      <c r="AA11" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="AB11" t="inlineStr">
+        <is>
+          <t>हस्ताक्षर लिये गये हैं</t>
+        </is>
+      </c>
+      <c r="AC11" t="inlineStr">
+        <is>
+          <t>चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।</t>
+        </is>
+      </c>
+      <c r="AD11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","v_name":"भिनाय","v_khata":"0","v_khasra":"0","v_area":"0","v_lagan":"0","v_cultivable":"0","v_sivaychak":"0","v_pasture":"0"}]</t>
+        </is>
+      </c>
+      <c r="AK11" t="inlineStr">
+        <is>
+          <t>गत निरीक्षण के निर्देशों की पालना की जा चुकी है।</t>
+        </is>
+      </c>
+      <c r="AL11" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"","ins_officer":"तहसीलदार भिनाय","ins_date":"2025-10-15","ins_receive_date":"2025-10-20","ins_compliance_date":"2025-10-25"}],"remarks":"गत निरीक्षण के निर्देशों की पालना की जा चुकी है।"}</t>
+        </is>
+      </c>
+      <c r="AM11" t="inlineStr">
+        <is>
+          <t>{"diary_pages":"हाँ","diary_blank_pages":"हाँ","diary_certified":"हाँ","diary_period":"हाँ","diary_extraordinary":"लागू नहीं","diary_govt_work":"हाँ","diary_recovery":"हाँ","diary_annual_reg":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="AN11" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","map_jamabandi":"0","map_sheet1":"0","map_sheet2":"0","map_diff_reason":"कोई अन्तर नहीं"}],"remarks":"जमाबंदी व नक्शा खसरा मिलान में कोई महत्वपूर्ण अन्तर नहीं पाया गया।"}</t>
+        </is>
+      </c>
+      <c r="AO11" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","g_samvat":"2082","g_rotation":"","g_crop":"","g_goswara":"अंकित","g_kharaba":"नहीं","g_trees":"नहीं","g_encroach":"नहीं","g_zero":"नहीं"}],"remarks":"निर्धारित प्रपत्र में संधारित की जा रही है/ऑनलाइन की जा रही है"}</t>
+        </is>
+      </c>
+      <c r="AP11" t="inlineStr">
+        <is>
+          <t>["जांच की गई","जांच की गई","इन्द्राज पूर्ण","विवरण अंकित","रिपोर्ट समय पर प्रेषित","पूर्ति की गई"]</t>
+        </is>
+      </c>
+      <c r="AQ11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","e_sivay_count":"0","e_past_count":"0","e_sivay_check":"जांच की गई","e_past_check":"जांच की गई","e_sivay_enc":"0","e_past_enc":"0","e_report_time":"समय पर","e_report_delay":"समय पर"}]</t>
+        </is>
+      </c>
+      <c r="AR11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","p14_count":"0","p14_report":"लागू नहीं","p14_orders":"लागू नहीं","p14_eviction":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="AS11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","r91_status":"हाँ","r91_complete":"पूर्ण","r91_jinswar_detail":"हाँ","r91_remarks":"सुरक्षित"}]</t>
+        </is>
+      </c>
+      <c r="AT11" t="inlineStr">
+        <is>
+          <t>{"भिनाय":{"खरीफ पी-16":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"रबी पी-17":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"जायद रबी पी-18":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"मिलान खसरा पी-19":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"पूरक मिलान खसरा पी-19क":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false}}}</t>
+        </is>
+      </c>
+      <c r="AU11" t="inlineStr">
+        <is>
+          <t>{"village_table":[{"v_sync_name":"भिनाय","mu_filed":"0","mu_decided":"0","mu_pending":"0","mu_decision_sheet":"0","mu_execution":"पूर्ण","mu_period":"लागू नहीं","mu_reason":"लागू नहीं"}],"levels_table":[{"ml_level_name":"पटवारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"एलआरसी (LRC) स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"भू-अभिलेख निरीक्षक स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"राजस्व अधिकारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"पंचायत स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"निषेधाज्ञा से अवशेष","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""}],"types_table":[{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"शुद्धिपत्र","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"हकतर्कनामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहननामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहनफक","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"बेचान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"दान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"वसीयत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"न्यायालय आदेश","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"स्थगन नोट","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"सहमति विभाजन","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"समर्पण","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"विरासत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"अन्य","mtype_doc_status":"संलग्न है","mtype_remarks":""}],"sec_12_4":{"mut_illegal":"कोई नहीं","mut_duplicate":"कोई नहीं","mut_reference":"कोई नहीं","mut_blank":"कोई नहीं","mut_glmac":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="AV11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","sh_decided":"0","sh_docs":"पूर्ण है","sh_remarks":"पूर्ण"}]</t>
+        </is>
+      </c>
+      <c r="AW11" t="inlineStr">
+        <is>
+          <t>{"tableA":[{"v_sync_name":"भिनाय","db_khata":"0","db_write":"0","db_check":"0","db_tra":"0","db_pending":"0"}],"tableB":[{"v_sync_name":"भिनाय","db_b_khata":"0","db_b_patwari":"0","db_b_ilr":"0","db_b_tra":"0","db_b_officer":"0","db_b_reason":"लागू नहीं"}],"rule107_remarks":"मांग पत्र नियमानुसार तैयार कर भू-अभिलेख निरीक्षक को प्रेषित किया गया है।","pending_cases":[{"v_sync_name":"भिनाय","pc_total_apps":"0","pc_disposed_apps":"0","pc_pending_apps":"0","pc_patwari_pending":"0","pc_tehsildar_pending":"0","pc_30days_pending":"0"}]}</t>
+        </is>
+      </c>
+      <c r="AX11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","rec_head":"भू-राजस्व","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"विविध","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"सिंचाई","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"नहर","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अति0 लगान","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अन्य","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AY11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","tr_head":"भू-राजस्व","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"विविध","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"सिंचाई","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"नहर","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अति0 लगान","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अन्य","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AZ11" t="inlineStr">
+        <is>
+          <t>{"copy_reg_status":"हाँ","copy_total_issued":"0","copy_pending_apps":"0","copy_fee_deposited":"हाँ","copy_serial_order":"हाँ","copy_fee_serial":"0","copy_fee_amount":"0","copy_fee_words":"शून्य","copy_monthly_meeting_deposit":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="BA11" t="inlineStr">
+        <is>
+          <t>{"store_reg_status":"हाँ","store_verification_date":"2026-04-10","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37":{"p37_reg_status":"हाँ","p37_unavailable_samvat":"लागू नहीं","p37_submitted_upto":"2080","p37_pending_samvat":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="BB11" t="inlineStr">
+        <is>
+          <t>{"passbook_total_holders":"0","passbook_total_dist":"0","passbook_pending":"0","passbook_completed":"0","passbook_fee_status":"पासबुकों का राजकीय शुल्क जमा करा दिया गया है"}</t>
+        </is>
+      </c>
+      <c r="BC11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","nk_custodian":"0","nk_allottee":"0","nk_settled":"0","nk_leaseholder":"0"}]</t>
+        </is>
+      </c>
+      <c r="BD11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cv_khasra":"कोई नहीं","cv_purpose":"लागू नहीं","cv_action":"लागू नहीं","cv_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BE11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cc_order_date":"लागू नहीं","cc_purpose":"लागू नहीं","cc_actual":"लागू नहीं","cc_action":"लागू नहीं","cc_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BF11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cm_order_date":"लागू नहीं","cm_entry":"लागू नहीं","cm_sale":"लागू नहीं","cm_mutation":"लागू नहीं","cm_others":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BG11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","al_order_date":"लागू नहीं","al_purpose":"लागू नहीं","al_actual":"लागू नहीं","al_action":"लागू नहीं","al_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BH11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","ga_offices":"0","ga_cases":"0","ga_pending":"0","ga_private":"0","ga_diff":"0"}]</t>
+        </is>
+      </c>
+      <c r="BI11" t="inlineStr">
+        <is>
+          <t>{"seeding":[{"v_sync_name":"भिनाय","sd_ver_pending":"0","sd_land":"0","sd_aadhaar":"0"}],"znms":[{"v_sync_name":"भिनाय","zn_draft":"0","zn_ver":"0","zn_znms":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BJ11" t="inlineStr">
+        <is>
+          <t>{"relief":[{"v_sync_name":"भिनाय","di_fire":"0","di_flood":"0","di_house":"0","di_lightning":"0","di_others":"0"}],"accidents":[{"v_sync_name":"भिनाय","ac_accident":"0","ac_drown":"0","ac_elec":"0","ac_collapse":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BK11" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","bs_total":"0","bs_bank":"0","bs_aadhaar":"0","bs_errors":"0"}]</t>
+        </is>
+      </c>
+      <c r="BL11" t="inlineStr">
+        <is>
+          <t>{"rule116_status":"संधारित है","rule116_sign":"हस्ताक्षर लिये गये हैं","rule117_egras":"चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।","copy_reg_status":"हाँ","store_reg_status":"हाँ","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37_reg_status":"हाँ","passbook_total_dist":"0","seeding_remarks":"पीएम किसान योजना के अंतर्गत सीडिंग व फार्मर रजिस्ट्री का कार्य लगभग पूर्ण हो चुका है।","r91_active_count":"1","r91_inactive_count":"0","r91_overall_remarks":"सीमा चिन्ह सुरक्षित अवस्था में हैं तथा सीमांकन रजिस्टर पूर्ण है।","jinswar_remarks":"सामयिक फसल विवरण पत्र (जिंसवार) समय पर प्रस्तुत किए गए हैं।","rule121_pending_date":"","copy_remarks":"नकल पंजिका पूर्ण व अद्यतन है, राजकीय शुल्क समय पर जमा है।","store_remarks":"सर्वे यंत्र पंजिका पूर्ण व अद्यतन है।","passbook_remarks":"कृषि जोत पासबुक का अधिकांश वितरण पूर्ण हो चुका है, शेष प्रगति पर है।","r89_register_status":"संधारित की जा रही है","check_girdawari_remarks":"नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।","dhal_samvat":"2081","dhal_year":"2024","recovery_not_started_count":"0","recovery_last_date":"2026-05-31","recovery_pending_start_date":"2026-04-01","recovery_pending_end_date":"2026-05-31","seamaprakaran_total_pending":"0","seamaprakaran_remarks":"लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।","citizen_charter_register_status":"नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।","grievances_register_status":"अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।","rti_register_status":"सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।","govt_schemes_progress":"राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।","conclusion_text":"","sdm_dispatch_no":"","sdm_dispatch_date":"","sdm_dispatch_tehsil":"","sdm_dispatch_patwari_circle":"","sdm_dispatch_patwari_tehsil":"","cv_remarks":"कृषि भूमि का विधि विपरीत अकृषि उपयोग का कोई नवीन प्रकरण ध्यान में नहीं आया है।","cc_remarks":"रूपांतरित भूमि का उपयोग स्वीकृत प्रयोजनार्थ ही किया जा रहा है।","al_remarks":"राजकीय प्रयोजनार्थ आवंटित भूमि का उपयोग संबंधित विभागों द्वारा नियमानुसार किया जा रहा है।","ga_remarks":"राजकीय कार्यालयों को आवंटित भूमियों का रिकॉर्ड में नियमानुसार अमल दर्ज है।","court_cases_remarks":"बकाया वसूली प्रकरणों में कुर्की व नीलामी की कार्रवाई प्रगति पर है।","nk_inst_custodian":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_allottee":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_settled":"बंदोबस्त रिकॉर्ड अनुसार खातेदारी अधिकार दिए गए हैं।","nk_inst_leaseholder":"लीज शर्तो की पालना सुनिश्चित की जा रही है।","exam_passed_year":"2015","dhal_remarks":"ढालबांछों का मिलान व प्रमाणीकरण समय पर पूर्ण किया गया है।","recovery_remarks":"राजस्व वसूली नियमित रूप से कर राजकोष में जमा कराई जा रही है।","rule116_remarks":"काश्तकारों को रसीदें प्रदान कर उनके हस्ताक्षर लिए गए हैं।","accidents_remarks":"दुर्घटना/डूबने/विद्युत आपदा राहत के सभी प्रकरणों में समय पर सहायता राशि स्वीकृत कराई गई है।","diary_duty_compliance":"हाँ","diary_duty_remarks":"पालना की जा रही है","jinswar_submit_status":"समय पर पेश किये जाते हैं"}</t>
+        </is>
+      </c>
+      <c r="BM11" t="inlineStr">
+        <is>
+          <t>{"summary":{"mact":"0","lr":"0","pdr":"0","irr":"0","audit":"0"},"cases":[{"type":"MACT","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"LR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"PDR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"IRR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"Audit","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""}]}</t>
+        </is>
+      </c>
+      <c r="BT11" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="BU11" t="inlineStr">
+        <is>
+          <t>{"pending":[{"p_sec_name":"111, 128","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"131","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"136","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"53","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"88","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"251ए","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"188","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"अन्य","p_sec_count":"0","p_sec_period":"0"}],"decided":[{"d_sec_name":"111, 128","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"131","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"136","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"53","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"88","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"251ए","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"188","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"अन्य","d_sec_count":"0","d_sec_period":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BV11" t="inlineStr">
+        <is>
+          <t>[{"v_name":"भिनाय","double_tenant":0,"blank_accounts":0,"adjacent_khasras":0,"no_share":0,"minor_guardian":0,"respectful_caste":0,"no_caste":0,"khatedar_nonkhatedar":0,"govt_pasture_mixed":0,"abadi_cremation_govt":0,"private_mortgage":0,"temple_mafi":0,"path_cremation_only":0,"no_conversion_govt":0,"adopted_son":0,"different_castes":0,"grandson_parentage":0,"deceased_inheritance":0,"conversion_purpose_mismatch":0,"no_separate_account":0,"school_playground_govt":0,"path_surrendered":0,"converted_in_zeroone":0,"other_corrections":0}]</t>
+        </is>
+      </c>
+      <c r="BW11" t="inlineStr">
+        <is>
+          <t>{"circ_1":"पूर्ण","circ_2":"हाँ","circ_3":"हाँ","circ_4":"125 दिनांक 15/05/2026","circ_5":"आदेश पुस्तक अद्यतन है।","circ_status":"बनी हुई है","circ_order_no":"125","circ_order_date":"2026-05-15","circ_order_subject":"राजस्व कार्य समीक्षा","remarks":"आदेश पंजिका में सभी महत्वपूर्ण आदेश अंकित हैं।"}</t>
+        </is>
+      </c>
+      <c r="BX11" t="inlineStr">
+        <is>
+          <t>{"remarks":"कोई विशेष कमी नहीं पाई गई।","status":"समय पर","jan":"2026-01-05","feb":"2026-02-05","mar":"2026-03-05","apr":"2026-04-05","may":"2026-05-05","jun":"2026-06-05","jul":"2026-07-05","aug":"2026-08-05","sep":"2026-09-05","oct":"2026-10-05","nov":"2026-11-05","dec":"2026-12-05"}</t>
+        </is>
+      </c>
+      <c r="BY11" t="inlineStr">
+        <is>
+          <t>नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।</t>
+        </is>
+      </c>
+      <c r="BZ11" t="inlineStr">
+        <is>
+          <t>अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।</t>
+        </is>
+      </c>
+      <c r="CA11" t="inlineStr">
+        <is>
+          <t>सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।</t>
+        </is>
+      </c>
+      <c r="CB11" t="inlineStr">
+        <is>
+          <t>राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।</t>
+        </is>
+      </c>
+      <c r="CC11" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="CD11" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="CS11" t="inlineStr">
+        <is>
+          <t>संधारित की जा रही है</t>
+        </is>
+      </c>
+      <c r="CT11" t="inlineStr">
+        <is>
+          <t>नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।</t>
+        </is>
+      </c>
+      <c r="CU11" t="inlineStr">
+        <is>
+          <t>2081</t>
+        </is>
+      </c>
+      <c r="CV11" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CW11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CX11" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="CY11" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="CZ11" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="DA11" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DB11" t="inlineStr">
+        <is>
+          <t>लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।</t>
+        </is>
+      </c>
+      <c r="DG11" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="DH11" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="DI11" t="inlineStr">
+        <is>
+          <t>पालना की जा रही है</t>
+        </is>
+      </c>
+      <c r="DJ11" t="inlineStr">
+        <is>
+          <t>समय पर पेश किये जाते हैं</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>REP-MOCK-20260610-2195</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>2026-06-10T22:11:12.044883</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>उपखंड अधिकारी भिनाय</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>1990-01-01</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t>स्नातक (Graduate)</t>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t>2015-08-15</t>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="P12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q12" t="inlineStr">
+        <is>
+          <t>स्थाई</t>
+        </is>
+      </c>
+      <c r="R12" t="inlineStr">
+        <is>
+          <t>प्रशिक्षित</t>
+        </is>
+      </c>
+      <c r="S12" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="T12" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="U12" t="inlineStr">
+        <is>
+          <t>सरकारी पटवार घर</t>
+        </is>
+      </c>
+      <c r="V12" t="inlineStr">
+        <is>
+          <t>तन्हा निवास</t>
+        </is>
+      </c>
+      <c r="W12" t="inlineStr">
+        <is>
+          <t>कोई नोटिस जारी नहीं।</t>
+        </is>
+      </c>
+      <c r="X12" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही विचाराधीन नहीं।</t>
+        </is>
+      </c>
+      <c r="Y12" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही निर्णित नहीं।</t>
+        </is>
+      </c>
+      <c r="AA12" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="AB12" t="inlineStr">
+        <is>
+          <t>हस्ताक्षर लिये गये हैं</t>
+        </is>
+      </c>
+      <c r="AC12" t="inlineStr">
+        <is>
+          <t>चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।</t>
+        </is>
+      </c>
+      <c r="AD12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","v_name":"भिनाय","v_khata":"0","v_khasra":"0","v_area":"0","v_lagan":"0","v_cultivable":"0","v_sivaychak":"0","v_pasture":"0"}]</t>
+        </is>
+      </c>
+      <c r="AK12" t="inlineStr">
+        <is>
+          <t>गत निरीक्षण के निर्देशों की पालना की जा चुकी है।</t>
+        </is>
+      </c>
+      <c r="AL12" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"","ins_officer":"तहसीलदार भिनाय","ins_date":"2025-10-15","ins_receive_date":"2025-10-20","ins_compliance_date":"2025-10-25"}],"remarks":"गत निरीक्षण के निर्देशों की पालना की जा चुकी है।"}</t>
+        </is>
+      </c>
+      <c r="AM12" t="inlineStr">
+        <is>
+          <t>{"diary_pages":"हाँ","diary_blank_pages":"हाँ","diary_certified":"हाँ","diary_period":"हाँ","diary_extraordinary":"लागू नहीं","diary_govt_work":"हाँ","diary_recovery":"हाँ","diary_annual_reg":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="AN12" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","map_jamabandi":"0","map_sheet1":"0","map_sheet2":"0","map_diff_reason":"कोई अन्तर नहीं"}],"remarks":"जमाबंदी व नक्शा खसरा मिलान में कोई महत्वपूर्ण अन्तर नहीं पाया गया।"}</t>
+        </is>
+      </c>
+      <c r="AO12" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","g_samvat":"2082","g_rotation":"","g_crop":"","g_goswara":"अंकित","g_kharaba":"नहीं","g_trees":"नहीं","g_encroach":"नहीं","g_zero":"नहीं"}],"remarks":"निर्धारित प्रपत्र में संधारित की जा रही है/ऑनलाइन की जा रही है"}</t>
+        </is>
+      </c>
+      <c r="AP12" t="inlineStr">
+        <is>
+          <t>["जांच की गई","जांच की गई","इन्द्राज पूर्ण","विवरण अंकित","रिपोर्ट समय पर प्रेषित","पूर्ति की गई"]</t>
+        </is>
+      </c>
+      <c r="AQ12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","e_sivay_count":"0","e_past_count":"0","e_sivay_check":"जांच की गई","e_past_check":"जांच की गई","e_sivay_enc":"0","e_past_enc":"0","e_report_time":"समय पर","e_report_delay":"समय पर"}]</t>
+        </is>
+      </c>
+      <c r="AR12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","p14_count":"0","p14_report":"लागू नहीं","p14_orders":"लागू नहीं","p14_eviction":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="AS12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","r91_status":"हाँ","r91_complete":"पूर्ण","r91_jinswar_detail":"हाँ","r91_remarks":"सुरक्षित"}]</t>
+        </is>
+      </c>
+      <c r="AT12" t="inlineStr">
+        <is>
+          <t>{"भिनाय":{"खरीफ पी-16":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"रबी पी-17":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"जायद रबी पी-18":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"मिलान खसरा पी-19":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"पूरक मिलान खसरा पी-19क":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false}}}</t>
+        </is>
+      </c>
+      <c r="AU12" t="inlineStr">
+        <is>
+          <t>{"village_table":[{"v_sync_name":"भिनाय","mu_filed":"0","mu_decided":"0","mu_pending":"0","mu_decision_sheet":"0","mu_execution":"पूर्ण","mu_period":"लागू नहीं","mu_reason":"लागू नहीं"}],"levels_table":[{"ml_level_name":"पटवारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"एलआरसी (LRC) स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"भू-अभिलेख निरीक्षक स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"राजस्व अधिकारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"पंचायत स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"निषेधाज्ञा से अवशेष","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""}],"types_table":[{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"शुद्धिपत्र","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"हकतर्कनामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहननामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहनफक","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"बेचान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"दान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"वसीयत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"न्यायालय आदेश","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"स्थगन नोट","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"सहमति विभाजन","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"समर्पण","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"विरासत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"अन्य","mtype_doc_status":"संलग्न है","mtype_remarks":""}],"sec_12_4":{"mut_illegal":"कोई नहीं","mut_duplicate":"कोई नहीं","mut_reference":"कोई नहीं","mut_blank":"कोई नहीं","mut_glmac":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="AV12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","sh_decided":"0","sh_docs":"पूर्ण है","sh_remarks":"पूर्ण"}]</t>
+        </is>
+      </c>
+      <c r="AW12" t="inlineStr">
+        <is>
+          <t>{"tableA":[{"v_sync_name":"भिनाय","db_khata":"0","db_write":"0","db_check":"0","db_tra":"0","db_pending":"0"}],"tableB":[{"v_sync_name":"भिनाय","db_b_khata":"0","db_b_patwari":"0","db_b_ilr":"0","db_b_tra":"0","db_b_officer":"0","db_b_reason":"लागू नहीं"}],"rule107_remarks":"मांग पत्र नियमानुसार तैयार कर भू-अभिलेख निरीक्षक को प्रेषित किया गया है।","pending_cases":[{"v_sync_name":"भिनाय","pc_total_apps":"0","pc_disposed_apps":"0","pc_pending_apps":"0","pc_patwari_pending":"0","pc_tehsildar_pending":"0","pc_30days_pending":"0"}]}</t>
+        </is>
+      </c>
+      <c r="AX12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","rec_head":"भू-राजस्व","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"विविध","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"सिंचाई","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"नहर","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अति0 लगान","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अन्य","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AY12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","tr_head":"भू-राजस्व","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"विविध","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"सिंचाई","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"नहर","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अति0 लगान","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अन्य","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AZ12" t="inlineStr">
+        <is>
+          <t>{"copy_reg_status":"हाँ","copy_total_issued":"0","copy_pending_apps":"0","copy_fee_deposited":"हाँ","copy_serial_order":"हाँ","copy_fee_serial":"0","copy_fee_amount":"0","copy_fee_words":"शून्य","copy_monthly_meeting_deposit":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="BA12" t="inlineStr">
+        <is>
+          <t>{"store_reg_status":"हाँ","store_verification_date":"2026-04-10","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37":{"p37_reg_status":"हाँ","p37_unavailable_samvat":"लागू नहीं","p37_submitted_upto":"2080","p37_pending_samvat":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="BB12" t="inlineStr">
+        <is>
+          <t>{"passbook_total_holders":"0","passbook_total_dist":"0","passbook_pending":"0","passbook_completed":"0","passbook_fee_status":"पासबुकों का राजकीय शुल्क जमा करा दिया गया है"}</t>
+        </is>
+      </c>
+      <c r="BC12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","nk_custodian":"0","nk_allottee":"0","nk_settled":"0","nk_leaseholder":"0"}]</t>
+        </is>
+      </c>
+      <c r="BD12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cv_khasra":"कोई नहीं","cv_purpose":"लागू नहीं","cv_action":"लागू नहीं","cv_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BE12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cc_order_date":"लागू नहीं","cc_purpose":"लागू नहीं","cc_actual":"लागू नहीं","cc_action":"लागू नहीं","cc_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BF12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cm_order_date":"लागू नहीं","cm_entry":"लागू नहीं","cm_sale":"लागू नहीं","cm_mutation":"लागू नहीं","cm_others":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BG12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","al_order_date":"लागू नहीं","al_purpose":"लागू नहीं","al_actual":"लागू नहीं","al_action":"लागू नहीं","al_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BH12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","ga_offices":"0","ga_cases":"0","ga_pending":"0","ga_private":"0","ga_diff":"0"}]</t>
+        </is>
+      </c>
+      <c r="BI12" t="inlineStr">
+        <is>
+          <t>{"seeding":[{"v_sync_name":"भिनाय","sd_ver_pending":"0","sd_land":"0","sd_aadhaar":"0"}],"znms":[{"v_sync_name":"भिनाय","zn_draft":"0","zn_ver":"0","zn_znms":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BJ12" t="inlineStr">
+        <is>
+          <t>{"relief":[{"v_sync_name":"भिनाय","di_fire":"0","di_flood":"0","di_house":"0","di_lightning":"0","di_others":"0"}],"accidents":[{"v_sync_name":"भिनाय","ac_accident":"0","ac_drown":"0","ac_elec":"0","ac_collapse":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BK12" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","bs_total":"0","bs_bank":"0","bs_aadhaar":"0","bs_errors":"0"}]</t>
+        </is>
+      </c>
+      <c r="BL12" t="inlineStr">
+        <is>
+          <t>{"rule116_status":"संधारित है","rule116_sign":"हस्ताक्षर लिये गये हैं","rule117_egras":"चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।","copy_reg_status":"हाँ","store_reg_status":"हाँ","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37_reg_status":"हाँ","passbook_total_dist":"0","seeding_remarks":"पीएम किसान योजना के अंतर्गत सीडिंग व फार्मर रजिस्ट्री का कार्य लगभग पूर्ण हो चुका है।","r91_active_count":"1","r91_inactive_count":"0","r91_overall_remarks":"सीमा चिन्ह सुरक्षित अवस्था में हैं तथा सीमांकन रजिस्टर पूर्ण है।","jinswar_remarks":"सामयिक फसल विवरण पत्र (जिंसवार) समय पर प्रस्तुत किए गए हैं।","rule121_pending_date":"","copy_remarks":"नकल पंजिका पूर्ण व अद्यतन है, राजकीय शुल्क समय पर जमा है।","store_remarks":"सर्वे यंत्र पंजिका पूर्ण व अद्यतन है।","passbook_remarks":"कृषि जोत पासबुक का अधिकांश वितरण पूर्ण हो चुका है, शेष प्रगति पर है।","r89_register_status":"संधारित की जा रही है","check_girdawari_remarks":"नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।","dhal_samvat":"2081","dhal_year":"2024","recovery_not_started_count":"0","recovery_last_date":"2026-05-31","recovery_pending_start_date":"2026-04-01","recovery_pending_end_date":"2026-05-31","seamaprakaran_total_pending":"0","seamaprakaran_remarks":"लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।","citizen_charter_register_status":"नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।","grievances_register_status":"अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।","rti_register_status":"सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।","govt_schemes_progress":"राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।","conclusion_text":"","sdm_dispatch_no":"","sdm_dispatch_date":"","sdm_dispatch_tehsil":"","sdm_dispatch_patwari_circle":"","sdm_dispatch_patwari_tehsil":"","cv_remarks":"कृषि भूमि का विधि विपरीत अकृषि उपयोग का कोई नवीन प्रकरण ध्यान में नहीं आया है।","cc_remarks":"रूपांतरित भूमि का उपयोग स्वीकृत प्रयोजनार्थ ही किया जा रहा है।","al_remarks":"राजकीय प्रयोजनार्थ आवंटित भूमि का उपयोग संबंधित विभागों द्वारा नियमानुसार किया जा रहा है।","ga_remarks":"राजकीय कार्यालयों को आवंटित भूमियों का रिकॉर्ड में नियमानुसार अमल दर्ज है।","court_cases_remarks":"बकाया वसूली प्रकरणों में कुर्की व नीलामी की कार्रवाई प्रगति पर है।","nk_inst_custodian":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_allottee":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_settled":"बंदोबस्त रिकॉर्ड अनुसार खातेदारी अधिकार दिए गए हैं।","nk_inst_leaseholder":"लीज शर्तो की पालना सुनिश्चित की जा रही है।","exam_passed_year":"2015","dhal_remarks":"ढालबांछों का मिलान व प्रमाणीकरण समय पर पूर्ण किया गया है।","recovery_remarks":"राजस्व वसूली नियमित रूप से कर राजकोष में जमा कराई जा रही है।","rule116_remarks":"काश्तकारों को रसीदें प्रदान कर उनके हस्ताक्षर लिए गए हैं।","accidents_remarks":"दुर्घटना/डूबने/विद्युत आपदा राहत के सभी प्रकरणों में समय पर सहायता राशि स्वीकृत कराई गई है।","diary_duty_compliance":"हाँ","diary_duty_remarks":"पालना की जा रही है","jinswar_submit_status":"समय पर पेश किये जाते हैं"}</t>
+        </is>
+      </c>
+      <c r="BM12" t="inlineStr">
+        <is>
+          <t>{"summary":{"mact":"0","lr":"0","pdr":"0","irr":"0","audit":"0"},"cases":[{"type":"MACT","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"LR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"PDR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"IRR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"Audit","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""}]}</t>
+        </is>
+      </c>
+      <c r="BT12" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="BU12" t="inlineStr">
+        <is>
+          <t>{"pending":[{"p_sec_name":"111, 128","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"131","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"136","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"53","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"88","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"251ए","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"188","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"अन्य","p_sec_count":"0","p_sec_period":"0"}],"decided":[{"d_sec_name":"111, 128","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"131","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"136","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"53","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"88","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"251ए","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"188","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"अन्य","d_sec_count":"0","d_sec_period":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BV12" t="inlineStr">
+        <is>
+          <t>[{"v_name":"भिनाय","double_tenant":0,"blank_accounts":0,"adjacent_khasras":0,"no_share":0,"minor_guardian":0,"respectful_caste":0,"no_caste":0,"khatedar_nonkhatedar":0,"govt_pasture_mixed":0,"abadi_cremation_govt":0,"private_mortgage":0,"temple_mafi":0,"path_cremation_only":0,"no_conversion_govt":0,"adopted_son":0,"different_castes":0,"grandson_parentage":0,"deceased_inheritance":0,"conversion_purpose_mismatch":0,"no_separate_account":0,"school_playground_govt":0,"path_surrendered":0,"converted_in_zeroone":0,"other_corrections":0}]</t>
+        </is>
+      </c>
+      <c r="BW12" t="inlineStr">
+        <is>
+          <t>{"circ_1":"पूर्ण","circ_2":"हाँ","circ_3":"हाँ","circ_4":"125 दिनांक 15/05/2026","circ_5":"आदेश पुस्तक अद्यतन है।","circ_status":"बनी हुई है","circ_order_no":"125","circ_order_date":"2026-05-15","circ_order_subject":"राजस्व कार्य समीक्षा","remarks":"आदेश पंजिका में सभी महत्वपूर्ण आदेश अंकित हैं।"}</t>
+        </is>
+      </c>
+      <c r="BX12" t="inlineStr">
+        <is>
+          <t>{"remarks":"कोई विशेष कमी नहीं पाई गई।","status":"समय पर","jan":"2026-01-05","feb":"2026-02-05","mar":"2026-03-05","apr":"2026-04-05","may":"2026-05-05","jun":"2026-06-05","jul":"2026-07-05","aug":"2026-08-05","sep":"2026-09-05","oct":"2026-10-05","nov":"2026-11-05","dec":"2026-12-05"}</t>
+        </is>
+      </c>
+      <c r="BY12" t="inlineStr">
+        <is>
+          <t>नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।</t>
+        </is>
+      </c>
+      <c r="BZ12" t="inlineStr">
+        <is>
+          <t>अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।</t>
+        </is>
+      </c>
+      <c r="CA12" t="inlineStr">
+        <is>
+          <t>सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।</t>
+        </is>
+      </c>
+      <c r="CB12" t="inlineStr">
+        <is>
+          <t>राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।</t>
+        </is>
+      </c>
+      <c r="CC12" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="CD12" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="CS12" t="inlineStr">
+        <is>
+          <t>संधारित की जा रही है</t>
+        </is>
+      </c>
+      <c r="CT12" t="inlineStr">
+        <is>
+          <t>नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।</t>
+        </is>
+      </c>
+      <c r="CU12" t="inlineStr">
+        <is>
+          <t>2081</t>
+        </is>
+      </c>
+      <c r="CV12" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CW12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CX12" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="CY12" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="CZ12" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="DA12" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DB12" t="inlineStr">
+        <is>
+          <t>लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।</t>
+        </is>
+      </c>
+      <c r="DG12" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="DH12" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="DI12" t="inlineStr">
+        <is>
+          <t>पालना की जा रही है</t>
+        </is>
+      </c>
+      <c r="DJ12" t="inlineStr">
+        <is>
+          <t>समय पर पेश किये जाते हैं</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>REP-MOCK-20260610-3464</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>2026-06-10T22:11:20.752528</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr"/>
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>उपखंड अधिकारी भिनाय</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr"/>
+      <c r="G13" t="inlineStr"/>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-06-10</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>1990-01-01</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t>अजमेर</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t>स्नातक (Graduate)</t>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t>2015-08-15</t>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t>2020-01-10</t>
+        </is>
+      </c>
+      <c r="P13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="Q13" t="inlineStr">
+        <is>
+          <t>स्थाई</t>
+        </is>
+      </c>
+      <c r="R13" t="inlineStr">
+        <is>
+          <t>प्रशिक्षित</t>
+        </is>
+      </c>
+      <c r="S13" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="T13" t="inlineStr">
+        <is>
+          <t>भिनाय</t>
+        </is>
+      </c>
+      <c r="U13" t="inlineStr">
+        <is>
+          <t>सरकारी पटवार घर</t>
+        </is>
+      </c>
+      <c r="V13" t="inlineStr">
+        <is>
+          <t>तन्हा निवास</t>
+        </is>
+      </c>
+      <c r="W13" t="inlineStr">
+        <is>
+          <t>कोई नोटिस जारी नहीं।</t>
+        </is>
+      </c>
+      <c r="X13" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही विचाराधीन नहीं।</t>
+        </is>
+      </c>
+      <c r="Y13" t="inlineStr">
+        <is>
+          <t>कोई कार्यवाही निर्णित नहीं।</t>
+        </is>
+      </c>
+      <c r="Z13" t="inlineStr"/>
+      <c r="AA13" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="AB13" t="inlineStr">
+        <is>
+          <t>हस्ताक्षर लिये गये हैं</t>
+        </is>
+      </c>
+      <c r="AC13" t="inlineStr">
+        <is>
+          <t>चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।</t>
+        </is>
+      </c>
+      <c r="AD13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AE13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AF13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AG13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AH13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AI13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="AJ13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","v_name":"भिनाय","v_khata":"0","v_khasra":"0","v_area":"0","v_lagan":"0","v_cultivable":"0","v_sivaychak":"0","v_pasture":"0"}]</t>
+        </is>
+      </c>
+      <c r="AK13" t="inlineStr">
+        <is>
+          <t>गत निरीक्षण के निर्देशों की पालना की जा चुकी है।</t>
+        </is>
+      </c>
+      <c r="AL13" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"","ins_officer":"तहसीलदार भिनाय","ins_date":"2025-10-15","ins_receive_date":"2025-10-20","ins_compliance_date":"2025-10-25"}],"remarks":"गत निरीक्षण के निर्देशों की पालना की जा चुकी है।"}</t>
+        </is>
+      </c>
+      <c r="AM13" t="inlineStr">
+        <is>
+          <t>{"diary_pages":"हाँ","diary_blank_pages":"हाँ","diary_certified":"हाँ","diary_period":"हाँ","diary_extraordinary":"लागू नहीं","diary_govt_work":"हाँ","diary_recovery":"हाँ","diary_annual_reg":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="AN13" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","map_jamabandi":"0","map_sheet1":"0","map_sheet2":"0","map_diff_reason":"कोई अन्तर नहीं"}],"remarks":"जमाबंदी व नक्शा खसरा मिलान में कोई महत्वपूर्ण अन्तर नहीं पाया गया।"}</t>
+        </is>
+      </c>
+      <c r="AO13" t="inlineStr">
+        <is>
+          <t>{"list":[{"v_sync_name":"भिनाय","g_samvat":"2082","g_rotation":"","g_crop":"","g_goswara":"अंकित","g_kharaba":"नहीं","g_trees":"नहीं","g_encroach":"नहीं","g_zero":"नहीं"}],"remarks":"निर्धारित प्रपत्र में संधारित की जा रही है/ऑनलाइन की जा रही है"}</t>
+        </is>
+      </c>
+      <c r="AP13" t="inlineStr">
+        <is>
+          <t>["जांच की गई","जांच की गई","इन्द्राज पूर्ण","विवरण अंकित","रिपोर्ट समय पर प्रेषित","पूर्ति की गई"]</t>
+        </is>
+      </c>
+      <c r="AQ13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","e_sivay_count":"0","e_past_count":"0","e_sivay_check":"जांच की गई","e_past_check":"जांच की गई","e_sivay_enc":"0","e_past_enc":"0","e_report_time":"समय पर","e_report_delay":"समय पर"}]</t>
+        </is>
+      </c>
+      <c r="AR13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","p14_count":"0","p14_report":"लागू नहीं","p14_orders":"लागू नहीं","p14_eviction":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="AS13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","r91_status":"हाँ","r91_complete":"पूर्ण","r91_jinswar_detail":"हाँ","r91_remarks":"सुरक्षित"}]</t>
+        </is>
+      </c>
+      <c r="AT13" t="inlineStr">
+        <is>
+          <t>{"भिनाय":{"खरीफ पी-16":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"रबी पी-17":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"जायद रबी पी-18":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"मिलान खसरा पी-19":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false},"पूरक मिलान खसरा पी-19क":{"non_trs_date":"","trs_date":"","non_trs_ontime":false,"trs_ontime":false,"non_trs_delayed":false,"trs_delayed":false}}}</t>
+        </is>
+      </c>
+      <c r="AU13" t="inlineStr">
+        <is>
+          <t>{"village_table":[{"v_sync_name":"भिनाय","mu_filed":"0","mu_decided":"0","mu_pending":"0","mu_decision_sheet":"0","mu_execution":"पूर्ण","mu_period":"लागू नहीं","mu_reason":"लागू नहीं"}],"levels_table":[{"ml_level_name":"पटवारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"एलआरसी (LRC) स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"भू-अभिलेख निरीक्षक स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"राजस्व अधिकारी स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"पंचायत स्तर पर","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""},{"ml_level_name":"निषेधाज्ञा से अवशेष","ml_prev_pending":"0","ml_filed":"","ml_total":"","ml_computerized":"","ml_pending":"","ml_pending_period":"","ml_pending_reason":""}],"types_table":[{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"शुद्धिपत्र","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"हकतर्कनामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहननामा","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"रहनफक","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"बेचान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"दान","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"वसीयत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"न्यायालय आदेश","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"स्थगन नोट","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"सहमति विभाजन","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"समर्पण","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"विरासत","mtype_doc_status":"संलग्न है","mtype_remarks":""},{"v_sync_name":"","mtype_village":"भिनाय","mtype_name":"अन्य","mtype_doc_status":"संलग्न है","mtype_remarks":""}],"sec_12_4":{"mut_illegal":"कोई नहीं","mut_duplicate":"कोई नहीं","mut_reference":"कोई नहीं","mut_blank":"कोई नहीं","mut_glmac":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="AV13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","sh_decided":"0","sh_docs":"पूर्ण है","sh_remarks":"पूर्ण"}]</t>
+        </is>
+      </c>
+      <c r="AW13" t="inlineStr">
+        <is>
+          <t>{"tableA":[{"v_sync_name":"भिनाय","db_khata":"0","db_write":"0","db_check":"0","db_tra":"0","db_pending":"0"}],"tableB":[{"v_sync_name":"भिनाय","db_b_khata":"0","db_b_patwari":"0","db_b_ilr":"0","db_b_tra":"0","db_b_officer":"0","db_b_reason":"लागू नहीं"}],"rule107_remarks":"मांग पत्र नियमानुसार तैयार कर भू-अभिलेख निरीक्षक को प्रेषित किया गया है।","pending_cases":[{"v_sync_name":"भिनाय","pc_total_apps":"0","pc_disposed_apps":"0","pc_pending_apps":"0","pc_patwari_pending":"0","pc_tehsildar_pending":"0","pc_30days_pending":"0"}]}</t>
+        </is>
+      </c>
+      <c r="AX13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","rec_head":"भू-राजस्व","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"विविध","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"सिंचाई","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"नहर","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अति0 लगान","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"},{"v_sync_name":"भिनाय","rec_head":"अन्य","rec_demand_old":"0","rec_demand":"0","rec_collection_old":"0","rec_collection":"0","rec_status":"नियमित है","rec_challan":"राजकोष में जमा","rec_challan_no":"चालान संख्या 01","rec_tra_recovery":"0","rec_total":"0","rec_chaspa":"हाँ","rec_match":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AY13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","tr_head":"भू-राजस्व","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"विविध","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"सिंचाई","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"नहर","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अति0 लगान","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"},{"v_sync_name":"भिनाय","tr_head":"अन्य","tr_period":"2024-25","tr_recovery":"0","tr_amount_date":"","tr_amount":"0","tr_timeliness":"अवधि में","tr_tehsil_date":"","tr_diary":"हाँ"}]</t>
+        </is>
+      </c>
+      <c r="AZ13" t="inlineStr">
+        <is>
+          <t>{"copy_reg_status":"हाँ","copy_total_issued":"0","copy_pending_apps":"0","copy_fee_deposited":"हाँ","copy_serial_order":"हाँ","copy_fee_serial":"0","copy_fee_amount":"0","copy_fee_words":"शून्य","copy_monthly_meeting_deposit":"हाँ"}</t>
+        </is>
+      </c>
+      <c r="BA13" t="inlineStr">
+        <is>
+          <t>{"store_reg_status":"हाँ","store_verification_date":"2026-04-10","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37":{"p37_reg_status":"हाँ","p37_unavailable_samvat":"लागू नहीं","p37_submitted_upto":"2080","p37_pending_samvat":"कोई नहीं"}}</t>
+        </is>
+      </c>
+      <c r="BB13" t="inlineStr">
+        <is>
+          <t>{"passbook_total_holders":"0","passbook_total_dist":"0","passbook_pending":"0","passbook_completed":"0","passbook_fee_status":"पासबुकों का राजकीय शुल्क जमा करा दिया गया है"}</t>
+        </is>
+      </c>
+      <c r="BC13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","nk_custodian":"0","nk_allottee":"0","nk_settled":"0","nk_leaseholder":"0"}]</t>
+        </is>
+      </c>
+      <c r="BD13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cv_khasra":"कोई नहीं","cv_purpose":"लागू नहीं","cv_action":"लागू नहीं","cv_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BE13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cc_order_date":"लागू नहीं","cc_purpose":"लागू नहीं","cc_actual":"लागू नहीं","cc_action":"लागू नहीं","cc_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BF13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","cm_order_date":"लागू नहीं","cm_entry":"लागू नहीं","cm_sale":"लागू नहीं","cm_mutation":"लागू नहीं","cm_others":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BG13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","al_order_date":"लागू नहीं","al_purpose":"लागू नहीं","al_actual":"लागू नहीं","al_action":"लागू नहीं","al_order":"लागू नहीं"}]</t>
+        </is>
+      </c>
+      <c r="BH13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","ga_offices":"0","ga_cases":"0","ga_pending":"0","ga_private":"0","ga_diff":"0"}]</t>
+        </is>
+      </c>
+      <c r="BI13" t="inlineStr">
+        <is>
+          <t>{"seeding":[{"v_sync_name":"भिनाय","sd_ver_pending":"0","sd_land":"0","sd_aadhaar":"0"}],"znms":[{"v_sync_name":"भिनाय","zn_draft":"0","zn_ver":"0","zn_znms":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BJ13" t="inlineStr">
+        <is>
+          <t>{"relief":[{"v_sync_name":"भिनाय","di_fire":"0","di_flood":"0","di_house":"0","di_lightning":"0","di_others":"0"}],"accidents":[{"v_sync_name":"भिनाय","ac_accident":"0","ac_drown":"0","ac_elec":"0","ac_collapse":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BK13" t="inlineStr">
+        <is>
+          <t>[{"v_sync_name":"भिनाय","bs_total":"0","bs_bank":"0","bs_aadhaar":"0","bs_errors":"0"}]</t>
+        </is>
+      </c>
+      <c r="BL13" t="inlineStr">
+        <is>
+          <t>{"rule116_status":"संधारित है","rule116_sign":"हस्ताक्षर लिये गये हैं","rule117_egras":"चालान ऑनलाइन ई-ग्रास द्वारा जमा किए जाते हैं।","copy_reg_status":"हाँ","store_reg_status":"हाँ","store_items_status":"सभी सर्वे यंत्र / आलात पटवारी के पास सुरक्षित व चालू स्थिति में उपलब्ध हैं।","p37_reg_status":"हाँ","passbook_total_dist":"0","seeding_remarks":"पीएम किसान योजना के अंतर्गत सीडिंग व फार्मर रजिस्ट्री का कार्य लगभग पूर्ण हो चुका है।","r91_active_count":"1","r91_inactive_count":"0","r91_overall_remarks":"सीमा चिन्ह सुरक्षित अवस्था में हैं तथा सीमांकन रजिस्टर पूर्ण है।","jinswar_remarks":"सामयिक फसल विवरण पत्र (जिंसवार) समय पर प्रस्तुत किए गए हैं।","rule121_pending_date":"","copy_remarks":"नकल पंजिका पूर्ण व अद्यतन है, राजकीय शुल्क समय पर जमा है।","store_remarks":"सर्वे यंत्र पंजिका पूर्ण व अद्यतन है।","passbook_remarks":"कृषि जोत पासबुक का अधिकांश वितरण पूर्ण हो चुका है, शेष प्रगति पर है।","r89_register_status":"संधारित की जा रही है","check_girdawari_remarks":"नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।","dhal_samvat":"2081","dhal_year":"2024","recovery_not_started_count":"0","recovery_last_date":"2026-05-31","recovery_pending_start_date":"2026-04-01","recovery_pending_end_date":"2026-05-31","seamaprakaran_total_pending":"0","seamaprakaran_remarks":"लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।","citizen_charter_register_status":"नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।","grievances_register_status":"अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।","rti_register_status":"सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।","govt_schemes_progress":"राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।","conclusion_text":"","sdm_dispatch_no":"","sdm_dispatch_date":"","sdm_dispatch_tehsil":"","sdm_dispatch_patwari_circle":"","sdm_dispatch_patwari_tehsil":"","cv_remarks":"कृषि भूमि का विधि विपरीत अकृषि उपयोग का कोई नवीन प्रकरण ध्यान में नहीं आया है।","cc_remarks":"रूपांतरित भूमि का उपयोग स्वीकृत प्रयोजनार्थ ही किया जा रहा है।","al_remarks":"राजकीय प्रयोजनार्थ आवंटित भूमि का उपयोग संबंधित विभागों द्वारा नियमानुसार किया जा रहा है।","ga_remarks":"राजकीय कार्यालयों को आवंटित भूमियों का रिकॉर्ड में नियमानुसार अमल दर्ज है।","court_cases_remarks":"बकाया वसूली प्रकरणों में कुर्की व नीलामी की कार्रवाई प्रगति पर है।","nk_inst_custodian":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_allottee":"खातेदारी अधिकार प्रदायगी की कार्रवाई प्रक्रियाधीन है।","nk_inst_settled":"बंदोबस्त रिकॉर्ड अनुसार खातेदारी अधिकार दिए गए हैं।","nk_inst_leaseholder":"लीज शर्तो की पालना सुनिश्चित की जा रही है।","exam_passed_year":"2015","dhal_remarks":"ढालबांछों का मिलान व प्रमाणीकरण समय पर पूर्ण किया गया है।","recovery_remarks":"राजस्व वसूली नियमित रूप से कर राजकोष में जमा कराई जा रही है।","rule116_remarks":"काश्तकारों को रसीदें प्रदान कर उनके हस्ताक्षर लिए गए हैं।","accidents_remarks":"दुर्घटना/डूबने/विद्युत आपदा राहत के सभी प्रकरणों में समय पर सहायता राशि स्वीकृत कराई गई है।","diary_duty_compliance":"हाँ","diary_duty_remarks":"पालना की जा रही है","jinswar_submit_status":"समय पर पेश किये जाते हैं"}</t>
+        </is>
+      </c>
+      <c r="BM13" t="inlineStr">
+        <is>
+          <t>{"summary":{"mact":"0","lr":"0","pdr":"0","irr":"0","audit":"0"},"cases":[{"type":"MACT","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"LR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"PDR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"IRR","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""},{"type":"Audit","notice_date":"","served_date":"","report_date":"","kurki_date":"","compliance_date":"","auction_date":"","conclusion":""}]}</t>
+        </is>
+      </c>
+      <c r="BO13" t="inlineStr"/>
+      <c r="BP13" t="inlineStr"/>
+      <c r="BQ13" t="inlineStr"/>
+      <c r="BR13" t="inlineStr"/>
+      <c r="BS13" t="inlineStr"/>
+      <c r="BT13" t="inlineStr">
+        <is>
+          <t>Pending</t>
+        </is>
+      </c>
+      <c r="BU13" t="inlineStr">
+        <is>
+          <t>{"pending":[{"p_sec_name":"111, 128","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"131","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"136","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"53","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"88","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"251ए","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"188","p_sec_count":"0","p_sec_period":"0"},{"p_sec_name":"अन्य","p_sec_count":"0","p_sec_period":"0"}],"decided":[{"d_sec_name":"111, 128","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"131","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"136","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"53","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"88","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"251ए","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"188","d_sec_count":"0","d_sec_period":"0"},{"d_sec_name":"अन्य","d_sec_count":"0","d_sec_period":"0"}]}</t>
+        </is>
+      </c>
+      <c r="BV13" t="inlineStr">
+        <is>
+          <t>[{"v_name":"भिनाय","double_tenant":0,"blank_accounts":0,"adjacent_khasras":0,"no_share":0,"minor_guardian":0,"respectful_caste":0,"no_caste":0,"khatedar_nonkhatedar":0,"govt_pasture_mixed":0,"abadi_cremation_govt":0,"private_mortgage":0,"temple_mafi":0,"path_cremation_only":0,"no_conversion_govt":0,"adopted_son":0,"different_castes":0,"grandson_parentage":0,"deceased_inheritance":0,"conversion_purpose_mismatch":0,"no_separate_account":0,"school_playground_govt":0,"path_surrendered":0,"converted_in_zeroone":0,"other_corrections":0}]</t>
+        </is>
+      </c>
+      <c r="BW13" t="inlineStr">
+        <is>
+          <t>{"circ_1":"पूर्ण","circ_2":"हाँ","circ_3":"हाँ","circ_4":"125 दिनांक 15/05/2026","circ_5":"आदेश पुस्तक अद्यतन है।","circ_status":"बनी हुई है","circ_order_no":"125","circ_order_date":"2026-05-15","circ_order_subject":"राजस्व कार्य समीक्षा","remarks":"आदेश पंजिका में सभी महत्वपूर्ण आदेश अंकित हैं।"}</t>
+        </is>
+      </c>
+      <c r="BX13" t="inlineStr">
+        <is>
+          <t>{"remarks":"कोई विशेष कमी नहीं पाई गई।","status":"समय पर","jan":"2026-01-05","feb":"2026-02-05","mar":"2026-03-05","apr":"2026-04-05","may":"2026-05-05","jun":"2026-06-05","jul":"2026-07-05","aug":"2026-08-05","sep":"2026-09-05","oct":"2026-10-05","nov":"2026-11-05","dec":"2026-12-05"}</t>
+        </is>
+      </c>
+      <c r="BY13" t="inlineStr">
+        <is>
+          <t>नागरिक अधिकार पत्र पंजिका संधारित है तथा सभी आवेदन समय सीमा में निस्तारित हैं।</t>
+        </is>
+      </c>
+      <c r="BZ13" t="inlineStr">
+        <is>
+          <t>अभाव अभियोग पंजिका संधारित है, कोई शिकायत लंबित नहीं है।</t>
+        </is>
+      </c>
+      <c r="CA13" t="inlineStr">
+        <is>
+          <t>सूचना अधिकार पंजिका संधारित है, सभी आवेदनों का समय पर निस्तारण किया गया है।</t>
+        </is>
+      </c>
+      <c r="CB13" t="inlineStr">
+        <is>
+          <t>राज्य व केंद्र सरकार की कल्याणकारी योजनाओं (यथा पीएम-किसान) में प्रगति उत्कृष्ट है।</t>
+        </is>
+      </c>
+      <c r="CC13" t="inlineStr">
+        <is>
+          <t>संधारित है</t>
+        </is>
+      </c>
+      <c r="CD13" t="inlineStr">
+        <is>
+          <t>2026-06-01</t>
+        </is>
+      </c>
+      <c r="CQ13" t="inlineStr"/>
+      <c r="CR13" t="inlineStr"/>
+      <c r="CS13" t="inlineStr">
+        <is>
+          <t>संधारित की जा रही है</t>
+        </is>
+      </c>
+      <c r="CT13" t="inlineStr">
+        <is>
+          <t>नियमित जांच गिरदावरी की गई, कोई गंभीर त्रुटि नहीं पाई गई।</t>
+        </is>
+      </c>
+      <c r="CU13" t="inlineStr">
+        <is>
+          <t>2081</t>
+        </is>
+      </c>
+      <c r="CV13" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
+      <c r="CW13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="CX13" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="CY13" t="inlineStr">
+        <is>
+          <t>2026-04-01</t>
+        </is>
+      </c>
+      <c r="CZ13" t="inlineStr">
+        <is>
+          <t>2026-05-31</t>
+        </is>
+      </c>
+      <c r="DA13" t="inlineStr">
+        <is>
+          <t>0</t>
+        </is>
+      </c>
+      <c r="DB13" t="inlineStr">
+        <is>
+          <t>लंबित सीमाज्ञान प्रकरणों का त्वरित निस्तारण किया जा रहा है।</t>
+        </is>
+      </c>
+      <c r="DC13" t="inlineStr"/>
+      <c r="DD13" t="inlineStr"/>
+      <c r="DE13" t="inlineStr"/>
+      <c r="DF13" t="inlineStr"/>
+      <c r="DG13" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="DH13" t="inlineStr">
+        <is>
+          <t>हाँ</t>
+        </is>
+      </c>
+      <c r="DI13" t="inlineStr">
+        <is>
+          <t>पालना की जा रही है</t>
+        </is>
+      </c>
+      <c r="DJ13" t="inlineStr">
         <is>
           <t>समय पर पेश किये जाते हैं</t>
         </is>

</xml_diff>